<commit_message>
etsy: autonomos sem cara de IA (status e recibos em palavras, textos simples, fotos novas)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DYz1Azd3FHBSgFnLhXfMUY
</commit_message>
<xml_diff>
--- a/etsy/freelancer/Freelancer-Tax-Tracker.xlsx
+++ b/etsy/freelancer/Freelancer-Tax-Tracker.xlsx
@@ -115,7 +115,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -124,8 +124,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F6F4EF"/>
-        <bgColor rgb="00F6F4EF"/>
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -138,12 +138,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F6F78"/>
         <bgColor rgb="001F6F78"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-        <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -181,16 +175,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D9D4C7"/>
+        <color rgb="00D5DBDB"/>
       </left>
       <right style="thin">
-        <color rgb="00D9D4C7"/>
+        <color rgb="00D5DBDB"/>
       </right>
       <top style="thin">
-        <color rgb="00D9D4C7"/>
+        <color rgb="00D5DBDB"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D9D4C7"/>
+        <color rgb="00D5DBDB"/>
       </bottom>
     </border>
   </borders>
@@ -202,29 +196,31 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="9" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="10" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="11" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="9" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="10" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="11" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="6" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -234,7 +230,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -770,7 +766,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Your freelance year at a glance</t>
+          <t>Freelance dashboard</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -785,7 +781,7 @@
       <c r="A3" s="1" t="n"/>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Only the Settings year counts. Paid income only.</t>
+          <t>Shows the year set in Settings, and only income that has been paid.</t>
         </is>
       </c>
       <c r="C3" s="1" t="n"/>
@@ -953,7 +949,7 @@
       </c>
       <c r="G10" s="1" t="n"/>
       <c r="H10" s="14">
-        <f>COUNTIFS(Income!$G$6:$G$305,"⚠*")&amp;" overdue invoice(s): "&amp;FIXED(SUMIFS(Income!$E$6:$E$305,Income!$G$6:$G$305,"⚠*"),2)</f>
+        <f>IF(COUNTIFS(Income!$G$6:$G$305,"Overdue*")=0,"No overdue invoices",IF(COUNTIFS(Income!$G$6:$G$305,"Overdue*")=1,"1 invoice is",COUNTIFS(Income!$G$6:$G$305,"Overdue*")&amp;" invoices are")&amp;" overdue: "&amp;FIXED(SUMIFS(Income!$E$6:$E$305,Income!$G$6:$G$305,"Overdue*"),2))</f>
         <v/>
       </c>
       <c r="I10" s="1" t="n"/>
@@ -983,7 +979,7 @@
       </c>
       <c r="G11" s="1" t="n"/>
       <c r="H11" s="15">
-        <f>COUNTIFS(Income!$G$6:$G$305,"Waiting*")&amp;" invoice(s) waiting: "&amp;FIXED(SUMIFS(Income!$E$6:$E$305,Income!$G$6:$G$305,"Waiting*"),2)</f>
+        <f>IF(COUNTIFS(Income!$G$6:$G$305,"Waiting*")=0,"No invoices waiting for payment",IF(COUNTIFS(Income!$G$6:$G$305,"Waiting*")=1,"1 invoice",COUNTIFS(Income!$G$6:$G$305,"Waiting*")&amp;" invoices")&amp;" waiting for payment: "&amp;FIXED(SUMIFS(Income!$E$6:$E$305,Income!$G$6:$G$305,"Waiting*"),2))</f>
         <v/>
       </c>
       <c r="I11" s="1" t="n"/>
@@ -1013,7 +1009,7 @@
       </c>
       <c r="G12" s="1" t="n"/>
       <c r="H12" s="15">
-        <f>COUNTIFS(Expenses!$B$6:$B$505,"&lt;&gt;",Expenses!$F$6:$F$505,"&lt;&gt;TRUE")&amp;" expense(s) without a receipt"</f>
+        <f>IF(COUNTIFS(Expenses!$B$6:$B$505,"&lt;&gt;",Expenses!$F$6:$F$505,"&lt;&gt;Yes")=0,"Every expense has a receipt",IF(COUNTIFS(Expenses!$B$6:$B$505,"&lt;&gt;",Expenses!$F$6:$F$505,"&lt;&gt;Yes")=1,"1 expense has",COUNTIFS(Expenses!$B$6:$B$505,"&lt;&gt;",Expenses!$F$6:$F$505,"&lt;&gt;Yes")&amp;" expenses have")&amp;" no receipt yet")</f>
         <v/>
       </c>
       <c r="I12" s="1" t="n"/>
@@ -1043,7 +1039,7 @@
       </c>
       <c r="G13" s="1" t="n"/>
       <c r="H13" s="16">
-        <f>"Tax set-aside progress: "&amp;IF(E7=0,"—",FIXED(MIN(1,F7/E7)*100,0)&amp;"%")</f>
+        <f>"Put aside for tax so far: "&amp;IF(E7=0,"nothing due yet",FIXED(MIN(1,F7/E7)*100,0)&amp;"% of the amount")</f>
         <v/>
       </c>
       <c r="I13" s="1" t="n"/>
@@ -1868,6 +1864,21 @@
       <c r="I79" s="1" t="n"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="H10">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>LEFT(H10,2)="No"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H11">
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>LEFT(H11,2)="No"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H12">
+    <cfRule type="expression" priority="3" dxfId="0">
+      <formula>LEFT(H12,5)="Every"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -2720,7 +2731,7 @@
         <v>46108</v>
       </c>
       <c r="G6" s="26">
-        <f>IF(OR(B6="",E6=""),"",IF(F6&lt;&gt;"","✓ Paid",IF(TODAY()-B6&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B6-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B6)&amp;" day(s)")))</f>
+        <f>IF(OR(B6="",E6=""),"",IF(F6&lt;&gt;"","Paid",IF((TODAY()-B6)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B6-Settings!$C$10)&amp;IF((TODAY()-B6-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B6)&amp;IF((TODAY()-B6)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H6" s="1" t="n"/>
@@ -2747,7 +2758,7 @@
         <v>46165</v>
       </c>
       <c r="G7" s="26">
-        <f>IF(OR(B7="",E7=""),"",IF(F7&lt;&gt;"","✓ Paid",IF(TODAY()-B7&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B7-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B7)&amp;" day(s)")))</f>
+        <f>IF(OR(B7="",E7=""),"",IF(F7&lt;&gt;"","Paid",IF((TODAY()-B7)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B7-Settings!$C$10)&amp;IF((TODAY()-B7-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B7)&amp;IF((TODAY()-B7)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H7" s="1" t="n"/>
@@ -2774,7 +2785,7 @@
         <v>46223</v>
       </c>
       <c r="G8" s="26">
-        <f>IF(OR(B8="",E8=""),"",IF(F8&lt;&gt;"","✓ Paid",IF(TODAY()-B8&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B8-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B8)&amp;" day(s)")))</f>
+        <f>IF(OR(B8="",E8=""),"",IF(F8&lt;&gt;"","Paid",IF((TODAY()-B8)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B8-Settings!$C$10)&amp;IF((TODAY()-B8-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B8)&amp;IF((TODAY()-B8)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H8" s="1" t="n"/>
@@ -2801,7 +2812,7 @@
         <v>46253</v>
       </c>
       <c r="G9" s="26">
-        <f>IF(OR(B9="",E9=""),"",IF(F9&lt;&gt;"","✓ Paid",IF(TODAY()-B9&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B9-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B9)&amp;" day(s)")))</f>
+        <f>IF(OR(B9="",E9=""),"",IF(F9&lt;&gt;"","Paid",IF((TODAY()-B9)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B9-Settings!$C$10)&amp;IF((TODAY()-B9-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B9)&amp;IF((TODAY()-B9)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H9" s="1" t="n"/>
@@ -2828,7 +2839,7 @@
         <v>46273</v>
       </c>
       <c r="G10" s="26">
-        <f>IF(OR(B10="",E10=""),"",IF(F10&lt;&gt;"","✓ Paid",IF(TODAY()-B10&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B10-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B10)&amp;" day(s)")))</f>
+        <f>IF(OR(B10="",E10=""),"",IF(F10&lt;&gt;"","Paid",IF((TODAY()-B10)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B10-Settings!$C$10)&amp;IF((TODAY()-B10-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B10)&amp;IF((TODAY()-B10)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H10" s="1" t="n"/>
@@ -2853,7 +2864,7 @@
       </c>
       <c r="F11" s="23" t="n"/>
       <c r="G11" s="26">
-        <f>IF(OR(B11="",E11=""),"",IF(F11&lt;&gt;"","✓ Paid",IF(TODAY()-B11&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B11-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B11)&amp;" day(s)")))</f>
+        <f>IF(OR(B11="",E11=""),"",IF(F11&lt;&gt;"","Paid",IF((TODAY()-B11)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B11-Settings!$C$10)&amp;IF((TODAY()-B11-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B11)&amp;IF((TODAY()-B11)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H11" s="1" t="n"/>
@@ -2878,7 +2889,7 @@
       </c>
       <c r="F12" s="23" t="n"/>
       <c r="G12" s="26">
-        <f>IF(OR(B12="",E12=""),"",IF(F12&lt;&gt;"","✓ Paid",IF(TODAY()-B12&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B12-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B12)&amp;" day(s)")))</f>
+        <f>IF(OR(B12="",E12=""),"",IF(F12&lt;&gt;"","Paid",IF((TODAY()-B12)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B12-Settings!$C$10)&amp;IF((TODAY()-B12-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B12)&amp;IF((TODAY()-B12)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H12" s="1" t="n"/>
@@ -2903,7 +2914,7 @@
       </c>
       <c r="F13" s="23" t="n"/>
       <c r="G13" s="26">
-        <f>IF(OR(B13="",E13=""),"",IF(F13&lt;&gt;"","✓ Paid",IF(TODAY()-B13&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B13-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B13)&amp;" day(s)")))</f>
+        <f>IF(OR(B13="",E13=""),"",IF(F13&lt;&gt;"","Paid",IF((TODAY()-B13)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B13-Settings!$C$10)&amp;IF((TODAY()-B13-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B13)&amp;IF((TODAY()-B13)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H13" s="1" t="n"/>
@@ -2916,7 +2927,7 @@
       <c r="E14" s="25" t="n"/>
       <c r="F14" s="23" t="n"/>
       <c r="G14" s="26">
-        <f>IF(OR(B14="",E14=""),"",IF(F14&lt;&gt;"","✓ Paid",IF(TODAY()-B14&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B14-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B14)&amp;" day(s)")))</f>
+        <f>IF(OR(B14="",E14=""),"",IF(F14&lt;&gt;"","Paid",IF((TODAY()-B14)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B14-Settings!$C$10)&amp;IF((TODAY()-B14-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B14)&amp;IF((TODAY()-B14)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H14" s="1" t="n"/>
@@ -2929,7 +2940,7 @@
       <c r="E15" s="25" t="n"/>
       <c r="F15" s="23" t="n"/>
       <c r="G15" s="26">
-        <f>IF(OR(B15="",E15=""),"",IF(F15&lt;&gt;"","✓ Paid",IF(TODAY()-B15&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B15-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B15)&amp;" day(s)")))</f>
+        <f>IF(OR(B15="",E15=""),"",IF(F15&lt;&gt;"","Paid",IF((TODAY()-B15)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B15-Settings!$C$10)&amp;IF((TODAY()-B15-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B15)&amp;IF((TODAY()-B15)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H15" s="1" t="n"/>
@@ -2942,7 +2953,7 @@
       <c r="E16" s="25" t="n"/>
       <c r="F16" s="23" t="n"/>
       <c r="G16" s="26">
-        <f>IF(OR(B16="",E16=""),"",IF(F16&lt;&gt;"","✓ Paid",IF(TODAY()-B16&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B16-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B16)&amp;" day(s)")))</f>
+        <f>IF(OR(B16="",E16=""),"",IF(F16&lt;&gt;"","Paid",IF((TODAY()-B16)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B16-Settings!$C$10)&amp;IF((TODAY()-B16-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B16)&amp;IF((TODAY()-B16)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H16" s="1" t="n"/>
@@ -2955,7 +2966,7 @@
       <c r="E17" s="25" t="n"/>
       <c r="F17" s="23" t="n"/>
       <c r="G17" s="26">
-        <f>IF(OR(B17="",E17=""),"",IF(F17&lt;&gt;"","✓ Paid",IF(TODAY()-B17&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B17-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B17)&amp;" day(s)")))</f>
+        <f>IF(OR(B17="",E17=""),"",IF(F17&lt;&gt;"","Paid",IF((TODAY()-B17)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B17-Settings!$C$10)&amp;IF((TODAY()-B17-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B17)&amp;IF((TODAY()-B17)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H17" s="1" t="n"/>
@@ -2968,7 +2979,7 @@
       <c r="E18" s="25" t="n"/>
       <c r="F18" s="23" t="n"/>
       <c r="G18" s="26">
-        <f>IF(OR(B18="",E18=""),"",IF(F18&lt;&gt;"","✓ Paid",IF(TODAY()-B18&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B18-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B18)&amp;" day(s)")))</f>
+        <f>IF(OR(B18="",E18=""),"",IF(F18&lt;&gt;"","Paid",IF((TODAY()-B18)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B18-Settings!$C$10)&amp;IF((TODAY()-B18-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B18)&amp;IF((TODAY()-B18)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H18" s="1" t="n"/>
@@ -2981,7 +2992,7 @@
       <c r="E19" s="25" t="n"/>
       <c r="F19" s="23" t="n"/>
       <c r="G19" s="26">
-        <f>IF(OR(B19="",E19=""),"",IF(F19&lt;&gt;"","✓ Paid",IF(TODAY()-B19&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B19-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B19)&amp;" day(s)")))</f>
+        <f>IF(OR(B19="",E19=""),"",IF(F19&lt;&gt;"","Paid",IF((TODAY()-B19)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B19-Settings!$C$10)&amp;IF((TODAY()-B19-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B19)&amp;IF((TODAY()-B19)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H19" s="1" t="n"/>
@@ -2994,7 +3005,7 @@
       <c r="E20" s="25" t="n"/>
       <c r="F20" s="23" t="n"/>
       <c r="G20" s="26">
-        <f>IF(OR(B20="",E20=""),"",IF(F20&lt;&gt;"","✓ Paid",IF(TODAY()-B20&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B20-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B20)&amp;" day(s)")))</f>
+        <f>IF(OR(B20="",E20=""),"",IF(F20&lt;&gt;"","Paid",IF((TODAY()-B20)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B20-Settings!$C$10)&amp;IF((TODAY()-B20-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B20)&amp;IF((TODAY()-B20)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H20" s="1" t="n"/>
@@ -3007,7 +3018,7 @@
       <c r="E21" s="25" t="n"/>
       <c r="F21" s="23" t="n"/>
       <c r="G21" s="26">
-        <f>IF(OR(B21="",E21=""),"",IF(F21&lt;&gt;"","✓ Paid",IF(TODAY()-B21&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B21-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B21)&amp;" day(s)")))</f>
+        <f>IF(OR(B21="",E21=""),"",IF(F21&lt;&gt;"","Paid",IF((TODAY()-B21)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B21-Settings!$C$10)&amp;IF((TODAY()-B21-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B21)&amp;IF((TODAY()-B21)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H21" s="1" t="n"/>
@@ -3020,7 +3031,7 @@
       <c r="E22" s="25" t="n"/>
       <c r="F22" s="23" t="n"/>
       <c r="G22" s="26">
-        <f>IF(OR(B22="",E22=""),"",IF(F22&lt;&gt;"","✓ Paid",IF(TODAY()-B22&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B22-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B22)&amp;" day(s)")))</f>
+        <f>IF(OR(B22="",E22=""),"",IF(F22&lt;&gt;"","Paid",IF((TODAY()-B22)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B22-Settings!$C$10)&amp;IF((TODAY()-B22-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B22)&amp;IF((TODAY()-B22)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H22" s="1" t="n"/>
@@ -3033,7 +3044,7 @@
       <c r="E23" s="25" t="n"/>
       <c r="F23" s="23" t="n"/>
       <c r="G23" s="26">
-        <f>IF(OR(B23="",E23=""),"",IF(F23&lt;&gt;"","✓ Paid",IF(TODAY()-B23&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B23-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B23)&amp;" day(s)")))</f>
+        <f>IF(OR(B23="",E23=""),"",IF(F23&lt;&gt;"","Paid",IF((TODAY()-B23)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B23-Settings!$C$10)&amp;IF((TODAY()-B23-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B23)&amp;IF((TODAY()-B23)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H23" s="1" t="n"/>
@@ -3046,7 +3057,7 @@
       <c r="E24" s="25" t="n"/>
       <c r="F24" s="23" t="n"/>
       <c r="G24" s="26">
-        <f>IF(OR(B24="",E24=""),"",IF(F24&lt;&gt;"","✓ Paid",IF(TODAY()-B24&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B24-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B24)&amp;" day(s)")))</f>
+        <f>IF(OR(B24="",E24=""),"",IF(F24&lt;&gt;"","Paid",IF((TODAY()-B24)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B24-Settings!$C$10)&amp;IF((TODAY()-B24-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B24)&amp;IF((TODAY()-B24)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H24" s="1" t="n"/>
@@ -3059,7 +3070,7 @@
       <c r="E25" s="25" t="n"/>
       <c r="F25" s="23" t="n"/>
       <c r="G25" s="26">
-        <f>IF(OR(B25="",E25=""),"",IF(F25&lt;&gt;"","✓ Paid",IF(TODAY()-B25&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B25-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B25)&amp;" day(s)")))</f>
+        <f>IF(OR(B25="",E25=""),"",IF(F25&lt;&gt;"","Paid",IF((TODAY()-B25)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B25-Settings!$C$10)&amp;IF((TODAY()-B25-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B25)&amp;IF((TODAY()-B25)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H25" s="1" t="n"/>
@@ -3072,7 +3083,7 @@
       <c r="E26" s="25" t="n"/>
       <c r="F26" s="23" t="n"/>
       <c r="G26" s="26">
-        <f>IF(OR(B26="",E26=""),"",IF(F26&lt;&gt;"","✓ Paid",IF(TODAY()-B26&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B26-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B26)&amp;" day(s)")))</f>
+        <f>IF(OR(B26="",E26=""),"",IF(F26&lt;&gt;"","Paid",IF((TODAY()-B26)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B26-Settings!$C$10)&amp;IF((TODAY()-B26-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B26)&amp;IF((TODAY()-B26)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H26" s="1" t="n"/>
@@ -3085,7 +3096,7 @@
       <c r="E27" s="25" t="n"/>
       <c r="F27" s="23" t="n"/>
       <c r="G27" s="26">
-        <f>IF(OR(B27="",E27=""),"",IF(F27&lt;&gt;"","✓ Paid",IF(TODAY()-B27&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B27-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B27)&amp;" day(s)")))</f>
+        <f>IF(OR(B27="",E27=""),"",IF(F27&lt;&gt;"","Paid",IF((TODAY()-B27)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B27-Settings!$C$10)&amp;IF((TODAY()-B27-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B27)&amp;IF((TODAY()-B27)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H27" s="1" t="n"/>
@@ -3098,7 +3109,7 @@
       <c r="E28" s="25" t="n"/>
       <c r="F28" s="23" t="n"/>
       <c r="G28" s="26">
-        <f>IF(OR(B28="",E28=""),"",IF(F28&lt;&gt;"","✓ Paid",IF(TODAY()-B28&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B28-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B28)&amp;" day(s)")))</f>
+        <f>IF(OR(B28="",E28=""),"",IF(F28&lt;&gt;"","Paid",IF((TODAY()-B28)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B28-Settings!$C$10)&amp;IF((TODAY()-B28-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B28)&amp;IF((TODAY()-B28)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H28" s="1" t="n"/>
@@ -3111,7 +3122,7 @@
       <c r="E29" s="25" t="n"/>
       <c r="F29" s="23" t="n"/>
       <c r="G29" s="26">
-        <f>IF(OR(B29="",E29=""),"",IF(F29&lt;&gt;"","✓ Paid",IF(TODAY()-B29&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B29-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B29)&amp;" day(s)")))</f>
+        <f>IF(OR(B29="",E29=""),"",IF(F29&lt;&gt;"","Paid",IF((TODAY()-B29)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B29-Settings!$C$10)&amp;IF((TODAY()-B29-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B29)&amp;IF((TODAY()-B29)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H29" s="1" t="n"/>
@@ -3124,7 +3135,7 @@
       <c r="E30" s="25" t="n"/>
       <c r="F30" s="23" t="n"/>
       <c r="G30" s="26">
-        <f>IF(OR(B30="",E30=""),"",IF(F30&lt;&gt;"","✓ Paid",IF(TODAY()-B30&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B30-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B30)&amp;" day(s)")))</f>
+        <f>IF(OR(B30="",E30=""),"",IF(F30&lt;&gt;"","Paid",IF((TODAY()-B30)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B30-Settings!$C$10)&amp;IF((TODAY()-B30-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B30)&amp;IF((TODAY()-B30)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H30" s="1" t="n"/>
@@ -3137,7 +3148,7 @@
       <c r="E31" s="25" t="n"/>
       <c r="F31" s="23" t="n"/>
       <c r="G31" s="26">
-        <f>IF(OR(B31="",E31=""),"",IF(F31&lt;&gt;"","✓ Paid",IF(TODAY()-B31&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B31-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B31)&amp;" day(s)")))</f>
+        <f>IF(OR(B31="",E31=""),"",IF(F31&lt;&gt;"","Paid",IF((TODAY()-B31)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B31-Settings!$C$10)&amp;IF((TODAY()-B31-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B31)&amp;IF((TODAY()-B31)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H31" s="1" t="n"/>
@@ -3150,7 +3161,7 @@
       <c r="E32" s="25" t="n"/>
       <c r="F32" s="23" t="n"/>
       <c r="G32" s="26">
-        <f>IF(OR(B32="",E32=""),"",IF(F32&lt;&gt;"","✓ Paid",IF(TODAY()-B32&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B32-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B32)&amp;" day(s)")))</f>
+        <f>IF(OR(B32="",E32=""),"",IF(F32&lt;&gt;"","Paid",IF((TODAY()-B32)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B32-Settings!$C$10)&amp;IF((TODAY()-B32-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B32)&amp;IF((TODAY()-B32)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H32" s="1" t="n"/>
@@ -3163,7 +3174,7 @@
       <c r="E33" s="25" t="n"/>
       <c r="F33" s="23" t="n"/>
       <c r="G33" s="26">
-        <f>IF(OR(B33="",E33=""),"",IF(F33&lt;&gt;"","✓ Paid",IF(TODAY()-B33&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B33-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B33)&amp;" day(s)")))</f>
+        <f>IF(OR(B33="",E33=""),"",IF(F33&lt;&gt;"","Paid",IF((TODAY()-B33)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B33-Settings!$C$10)&amp;IF((TODAY()-B33-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B33)&amp;IF((TODAY()-B33)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H33" s="1" t="n"/>
@@ -3176,7 +3187,7 @@
       <c r="E34" s="25" t="n"/>
       <c r="F34" s="23" t="n"/>
       <c r="G34" s="26">
-        <f>IF(OR(B34="",E34=""),"",IF(F34&lt;&gt;"","✓ Paid",IF(TODAY()-B34&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B34-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B34)&amp;" day(s)")))</f>
+        <f>IF(OR(B34="",E34=""),"",IF(F34&lt;&gt;"","Paid",IF((TODAY()-B34)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B34-Settings!$C$10)&amp;IF((TODAY()-B34-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B34)&amp;IF((TODAY()-B34)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H34" s="1" t="n"/>
@@ -3189,7 +3200,7 @@
       <c r="E35" s="25" t="n"/>
       <c r="F35" s="23" t="n"/>
       <c r="G35" s="26">
-        <f>IF(OR(B35="",E35=""),"",IF(F35&lt;&gt;"","✓ Paid",IF(TODAY()-B35&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B35-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B35)&amp;" day(s)")))</f>
+        <f>IF(OR(B35="",E35=""),"",IF(F35&lt;&gt;"","Paid",IF((TODAY()-B35)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B35-Settings!$C$10)&amp;IF((TODAY()-B35-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B35)&amp;IF((TODAY()-B35)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H35" s="1" t="n"/>
@@ -3202,7 +3213,7 @@
       <c r="E36" s="25" t="n"/>
       <c r="F36" s="23" t="n"/>
       <c r="G36" s="26">
-        <f>IF(OR(B36="",E36=""),"",IF(F36&lt;&gt;"","✓ Paid",IF(TODAY()-B36&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B36-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B36)&amp;" day(s)")))</f>
+        <f>IF(OR(B36="",E36=""),"",IF(F36&lt;&gt;"","Paid",IF((TODAY()-B36)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B36-Settings!$C$10)&amp;IF((TODAY()-B36-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B36)&amp;IF((TODAY()-B36)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H36" s="1" t="n"/>
@@ -3215,7 +3226,7 @@
       <c r="E37" s="25" t="n"/>
       <c r="F37" s="23" t="n"/>
       <c r="G37" s="26">
-        <f>IF(OR(B37="",E37=""),"",IF(F37&lt;&gt;"","✓ Paid",IF(TODAY()-B37&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B37-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B37)&amp;" day(s)")))</f>
+        <f>IF(OR(B37="",E37=""),"",IF(F37&lt;&gt;"","Paid",IF((TODAY()-B37)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B37-Settings!$C$10)&amp;IF((TODAY()-B37-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B37)&amp;IF((TODAY()-B37)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H37" s="1" t="n"/>
@@ -3228,7 +3239,7 @@
       <c r="E38" s="25" t="n"/>
       <c r="F38" s="23" t="n"/>
       <c r="G38" s="26">
-        <f>IF(OR(B38="",E38=""),"",IF(F38&lt;&gt;"","✓ Paid",IF(TODAY()-B38&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B38-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B38)&amp;" day(s)")))</f>
+        <f>IF(OR(B38="",E38=""),"",IF(F38&lt;&gt;"","Paid",IF((TODAY()-B38)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B38-Settings!$C$10)&amp;IF((TODAY()-B38-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B38)&amp;IF((TODAY()-B38)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H38" s="1" t="n"/>
@@ -3241,7 +3252,7 @@
       <c r="E39" s="25" t="n"/>
       <c r="F39" s="23" t="n"/>
       <c r="G39" s="26">
-        <f>IF(OR(B39="",E39=""),"",IF(F39&lt;&gt;"","✓ Paid",IF(TODAY()-B39&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B39-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B39)&amp;" day(s)")))</f>
+        <f>IF(OR(B39="",E39=""),"",IF(F39&lt;&gt;"","Paid",IF((TODAY()-B39)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B39-Settings!$C$10)&amp;IF((TODAY()-B39-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B39)&amp;IF((TODAY()-B39)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H39" s="1" t="n"/>
@@ -3254,7 +3265,7 @@
       <c r="E40" s="25" t="n"/>
       <c r="F40" s="23" t="n"/>
       <c r="G40" s="26">
-        <f>IF(OR(B40="",E40=""),"",IF(F40&lt;&gt;"","✓ Paid",IF(TODAY()-B40&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B40-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B40)&amp;" day(s)")))</f>
+        <f>IF(OR(B40="",E40=""),"",IF(F40&lt;&gt;"","Paid",IF((TODAY()-B40)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B40-Settings!$C$10)&amp;IF((TODAY()-B40-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B40)&amp;IF((TODAY()-B40)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H40" s="1" t="n"/>
@@ -3267,7 +3278,7 @@
       <c r="E41" s="25" t="n"/>
       <c r="F41" s="23" t="n"/>
       <c r="G41" s="26">
-        <f>IF(OR(B41="",E41=""),"",IF(F41&lt;&gt;"","✓ Paid",IF(TODAY()-B41&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B41-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B41)&amp;" day(s)")))</f>
+        <f>IF(OR(B41="",E41=""),"",IF(F41&lt;&gt;"","Paid",IF((TODAY()-B41)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B41-Settings!$C$10)&amp;IF((TODAY()-B41-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B41)&amp;IF((TODAY()-B41)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H41" s="1" t="n"/>
@@ -3280,7 +3291,7 @@
       <c r="E42" s="25" t="n"/>
       <c r="F42" s="23" t="n"/>
       <c r="G42" s="26">
-        <f>IF(OR(B42="",E42=""),"",IF(F42&lt;&gt;"","✓ Paid",IF(TODAY()-B42&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B42-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B42)&amp;" day(s)")))</f>
+        <f>IF(OR(B42="",E42=""),"",IF(F42&lt;&gt;"","Paid",IF((TODAY()-B42)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B42-Settings!$C$10)&amp;IF((TODAY()-B42-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B42)&amp;IF((TODAY()-B42)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H42" s="1" t="n"/>
@@ -3293,7 +3304,7 @@
       <c r="E43" s="25" t="n"/>
       <c r="F43" s="23" t="n"/>
       <c r="G43" s="26">
-        <f>IF(OR(B43="",E43=""),"",IF(F43&lt;&gt;"","✓ Paid",IF(TODAY()-B43&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B43-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B43)&amp;" day(s)")))</f>
+        <f>IF(OR(B43="",E43=""),"",IF(F43&lt;&gt;"","Paid",IF((TODAY()-B43)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B43-Settings!$C$10)&amp;IF((TODAY()-B43-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B43)&amp;IF((TODAY()-B43)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H43" s="1" t="n"/>
@@ -3306,7 +3317,7 @@
       <c r="E44" s="25" t="n"/>
       <c r="F44" s="23" t="n"/>
       <c r="G44" s="26">
-        <f>IF(OR(B44="",E44=""),"",IF(F44&lt;&gt;"","✓ Paid",IF(TODAY()-B44&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B44-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B44)&amp;" day(s)")))</f>
+        <f>IF(OR(B44="",E44=""),"",IF(F44&lt;&gt;"","Paid",IF((TODAY()-B44)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B44-Settings!$C$10)&amp;IF((TODAY()-B44-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B44)&amp;IF((TODAY()-B44)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H44" s="1" t="n"/>
@@ -3319,7 +3330,7 @@
       <c r="E45" s="25" t="n"/>
       <c r="F45" s="23" t="n"/>
       <c r="G45" s="26">
-        <f>IF(OR(B45="",E45=""),"",IF(F45&lt;&gt;"","✓ Paid",IF(TODAY()-B45&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B45-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B45)&amp;" day(s)")))</f>
+        <f>IF(OR(B45="",E45=""),"",IF(F45&lt;&gt;"","Paid",IF((TODAY()-B45)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B45-Settings!$C$10)&amp;IF((TODAY()-B45-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B45)&amp;IF((TODAY()-B45)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H45" s="1" t="n"/>
@@ -3332,7 +3343,7 @@
       <c r="E46" s="25" t="n"/>
       <c r="F46" s="23" t="n"/>
       <c r="G46" s="26">
-        <f>IF(OR(B46="",E46=""),"",IF(F46&lt;&gt;"","✓ Paid",IF(TODAY()-B46&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B46-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B46)&amp;" day(s)")))</f>
+        <f>IF(OR(B46="",E46=""),"",IF(F46&lt;&gt;"","Paid",IF((TODAY()-B46)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B46-Settings!$C$10)&amp;IF((TODAY()-B46-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B46)&amp;IF((TODAY()-B46)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H46" s="1" t="n"/>
@@ -3345,7 +3356,7 @@
       <c r="E47" s="25" t="n"/>
       <c r="F47" s="23" t="n"/>
       <c r="G47" s="26">
-        <f>IF(OR(B47="",E47=""),"",IF(F47&lt;&gt;"","✓ Paid",IF(TODAY()-B47&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B47-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B47)&amp;" day(s)")))</f>
+        <f>IF(OR(B47="",E47=""),"",IF(F47&lt;&gt;"","Paid",IF((TODAY()-B47)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B47-Settings!$C$10)&amp;IF((TODAY()-B47-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B47)&amp;IF((TODAY()-B47)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H47" s="1" t="n"/>
@@ -3358,7 +3369,7 @@
       <c r="E48" s="25" t="n"/>
       <c r="F48" s="23" t="n"/>
       <c r="G48" s="26">
-        <f>IF(OR(B48="",E48=""),"",IF(F48&lt;&gt;"","✓ Paid",IF(TODAY()-B48&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B48-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B48)&amp;" day(s)")))</f>
+        <f>IF(OR(B48="",E48=""),"",IF(F48&lt;&gt;"","Paid",IF((TODAY()-B48)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B48-Settings!$C$10)&amp;IF((TODAY()-B48-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B48)&amp;IF((TODAY()-B48)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H48" s="1" t="n"/>
@@ -3371,7 +3382,7 @@
       <c r="E49" s="25" t="n"/>
       <c r="F49" s="23" t="n"/>
       <c r="G49" s="26">
-        <f>IF(OR(B49="",E49=""),"",IF(F49&lt;&gt;"","✓ Paid",IF(TODAY()-B49&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B49-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B49)&amp;" day(s)")))</f>
+        <f>IF(OR(B49="",E49=""),"",IF(F49&lt;&gt;"","Paid",IF((TODAY()-B49)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B49-Settings!$C$10)&amp;IF((TODAY()-B49-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B49)&amp;IF((TODAY()-B49)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H49" s="1" t="n"/>
@@ -3384,7 +3395,7 @@
       <c r="E50" s="25" t="n"/>
       <c r="F50" s="23" t="n"/>
       <c r="G50" s="26">
-        <f>IF(OR(B50="",E50=""),"",IF(F50&lt;&gt;"","✓ Paid",IF(TODAY()-B50&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B50-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B50)&amp;" day(s)")))</f>
+        <f>IF(OR(B50="",E50=""),"",IF(F50&lt;&gt;"","Paid",IF((TODAY()-B50)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B50-Settings!$C$10)&amp;IF((TODAY()-B50-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B50)&amp;IF((TODAY()-B50)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H50" s="1" t="n"/>
@@ -3397,7 +3408,7 @@
       <c r="E51" s="25" t="n"/>
       <c r="F51" s="23" t="n"/>
       <c r="G51" s="26">
-        <f>IF(OR(B51="",E51=""),"",IF(F51&lt;&gt;"","✓ Paid",IF(TODAY()-B51&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B51-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B51)&amp;" day(s)")))</f>
+        <f>IF(OR(B51="",E51=""),"",IF(F51&lt;&gt;"","Paid",IF((TODAY()-B51)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B51-Settings!$C$10)&amp;IF((TODAY()-B51-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B51)&amp;IF((TODAY()-B51)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H51" s="1" t="n"/>
@@ -3410,7 +3421,7 @@
       <c r="E52" s="25" t="n"/>
       <c r="F52" s="23" t="n"/>
       <c r="G52" s="26">
-        <f>IF(OR(B52="",E52=""),"",IF(F52&lt;&gt;"","✓ Paid",IF(TODAY()-B52&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B52-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B52)&amp;" day(s)")))</f>
+        <f>IF(OR(B52="",E52=""),"",IF(F52&lt;&gt;"","Paid",IF((TODAY()-B52)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B52-Settings!$C$10)&amp;IF((TODAY()-B52-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B52)&amp;IF((TODAY()-B52)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H52" s="1" t="n"/>
@@ -3423,7 +3434,7 @@
       <c r="E53" s="25" t="n"/>
       <c r="F53" s="23" t="n"/>
       <c r="G53" s="26">
-        <f>IF(OR(B53="",E53=""),"",IF(F53&lt;&gt;"","✓ Paid",IF(TODAY()-B53&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B53-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B53)&amp;" day(s)")))</f>
+        <f>IF(OR(B53="",E53=""),"",IF(F53&lt;&gt;"","Paid",IF((TODAY()-B53)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B53-Settings!$C$10)&amp;IF((TODAY()-B53-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B53)&amp;IF((TODAY()-B53)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H53" s="1" t="n"/>
@@ -3436,7 +3447,7 @@
       <c r="E54" s="25" t="n"/>
       <c r="F54" s="23" t="n"/>
       <c r="G54" s="26">
-        <f>IF(OR(B54="",E54=""),"",IF(F54&lt;&gt;"","✓ Paid",IF(TODAY()-B54&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B54-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B54)&amp;" day(s)")))</f>
+        <f>IF(OR(B54="",E54=""),"",IF(F54&lt;&gt;"","Paid",IF((TODAY()-B54)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B54-Settings!$C$10)&amp;IF((TODAY()-B54-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B54)&amp;IF((TODAY()-B54)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H54" s="1" t="n"/>
@@ -3449,7 +3460,7 @@
       <c r="E55" s="25" t="n"/>
       <c r="F55" s="23" t="n"/>
       <c r="G55" s="26">
-        <f>IF(OR(B55="",E55=""),"",IF(F55&lt;&gt;"","✓ Paid",IF(TODAY()-B55&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B55-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B55)&amp;" day(s)")))</f>
+        <f>IF(OR(B55="",E55=""),"",IF(F55&lt;&gt;"","Paid",IF((TODAY()-B55)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B55-Settings!$C$10)&amp;IF((TODAY()-B55-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B55)&amp;IF((TODAY()-B55)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H55" s="1" t="n"/>
@@ -3462,7 +3473,7 @@
       <c r="E56" s="25" t="n"/>
       <c r="F56" s="23" t="n"/>
       <c r="G56" s="26">
-        <f>IF(OR(B56="",E56=""),"",IF(F56&lt;&gt;"","✓ Paid",IF(TODAY()-B56&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B56-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B56)&amp;" day(s)")))</f>
+        <f>IF(OR(B56="",E56=""),"",IF(F56&lt;&gt;"","Paid",IF((TODAY()-B56)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B56-Settings!$C$10)&amp;IF((TODAY()-B56-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B56)&amp;IF((TODAY()-B56)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H56" s="1" t="n"/>
@@ -3475,7 +3486,7 @@
       <c r="E57" s="25" t="n"/>
       <c r="F57" s="23" t="n"/>
       <c r="G57" s="26">
-        <f>IF(OR(B57="",E57=""),"",IF(F57&lt;&gt;"","✓ Paid",IF(TODAY()-B57&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B57-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B57)&amp;" day(s)")))</f>
+        <f>IF(OR(B57="",E57=""),"",IF(F57&lt;&gt;"","Paid",IF((TODAY()-B57)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B57-Settings!$C$10)&amp;IF((TODAY()-B57-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B57)&amp;IF((TODAY()-B57)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H57" s="1" t="n"/>
@@ -3488,7 +3499,7 @@
       <c r="E58" s="25" t="n"/>
       <c r="F58" s="23" t="n"/>
       <c r="G58" s="26">
-        <f>IF(OR(B58="",E58=""),"",IF(F58&lt;&gt;"","✓ Paid",IF(TODAY()-B58&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B58-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B58)&amp;" day(s)")))</f>
+        <f>IF(OR(B58="",E58=""),"",IF(F58&lt;&gt;"","Paid",IF((TODAY()-B58)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B58-Settings!$C$10)&amp;IF((TODAY()-B58-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B58)&amp;IF((TODAY()-B58)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H58" s="1" t="n"/>
@@ -3501,7 +3512,7 @@
       <c r="E59" s="25" t="n"/>
       <c r="F59" s="23" t="n"/>
       <c r="G59" s="26">
-        <f>IF(OR(B59="",E59=""),"",IF(F59&lt;&gt;"","✓ Paid",IF(TODAY()-B59&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B59-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B59)&amp;" day(s)")))</f>
+        <f>IF(OR(B59="",E59=""),"",IF(F59&lt;&gt;"","Paid",IF((TODAY()-B59)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B59-Settings!$C$10)&amp;IF((TODAY()-B59-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B59)&amp;IF((TODAY()-B59)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H59" s="1" t="n"/>
@@ -3514,7 +3525,7 @@
       <c r="E60" s="25" t="n"/>
       <c r="F60" s="23" t="n"/>
       <c r="G60" s="26">
-        <f>IF(OR(B60="",E60=""),"",IF(F60&lt;&gt;"","✓ Paid",IF(TODAY()-B60&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B60-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B60)&amp;" day(s)")))</f>
+        <f>IF(OR(B60="",E60=""),"",IF(F60&lt;&gt;"","Paid",IF((TODAY()-B60)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B60-Settings!$C$10)&amp;IF((TODAY()-B60-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B60)&amp;IF((TODAY()-B60)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H60" s="1" t="n"/>
@@ -3527,7 +3538,7 @@
       <c r="E61" s="25" t="n"/>
       <c r="F61" s="23" t="n"/>
       <c r="G61" s="26">
-        <f>IF(OR(B61="",E61=""),"",IF(F61&lt;&gt;"","✓ Paid",IF(TODAY()-B61&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B61-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B61)&amp;" day(s)")))</f>
+        <f>IF(OR(B61="",E61=""),"",IF(F61&lt;&gt;"","Paid",IF((TODAY()-B61)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B61-Settings!$C$10)&amp;IF((TODAY()-B61-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B61)&amp;IF((TODAY()-B61)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H61" s="1" t="n"/>
@@ -3540,7 +3551,7 @@
       <c r="E62" s="25" t="n"/>
       <c r="F62" s="23" t="n"/>
       <c r="G62" s="26">
-        <f>IF(OR(B62="",E62=""),"",IF(F62&lt;&gt;"","✓ Paid",IF(TODAY()-B62&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B62-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B62)&amp;" day(s)")))</f>
+        <f>IF(OR(B62="",E62=""),"",IF(F62&lt;&gt;"","Paid",IF((TODAY()-B62)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B62-Settings!$C$10)&amp;IF((TODAY()-B62-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B62)&amp;IF((TODAY()-B62)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H62" s="1" t="n"/>
@@ -3553,7 +3564,7 @@
       <c r="E63" s="25" t="n"/>
       <c r="F63" s="23" t="n"/>
       <c r="G63" s="26">
-        <f>IF(OR(B63="",E63=""),"",IF(F63&lt;&gt;"","✓ Paid",IF(TODAY()-B63&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B63-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B63)&amp;" day(s)")))</f>
+        <f>IF(OR(B63="",E63=""),"",IF(F63&lt;&gt;"","Paid",IF((TODAY()-B63)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B63-Settings!$C$10)&amp;IF((TODAY()-B63-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B63)&amp;IF((TODAY()-B63)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H63" s="1" t="n"/>
@@ -3566,7 +3577,7 @@
       <c r="E64" s="25" t="n"/>
       <c r="F64" s="23" t="n"/>
       <c r="G64" s="26">
-        <f>IF(OR(B64="",E64=""),"",IF(F64&lt;&gt;"","✓ Paid",IF(TODAY()-B64&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B64-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B64)&amp;" day(s)")))</f>
+        <f>IF(OR(B64="",E64=""),"",IF(F64&lt;&gt;"","Paid",IF((TODAY()-B64)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B64-Settings!$C$10)&amp;IF((TODAY()-B64-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B64)&amp;IF((TODAY()-B64)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H64" s="1" t="n"/>
@@ -3579,7 +3590,7 @@
       <c r="E65" s="25" t="n"/>
       <c r="F65" s="23" t="n"/>
       <c r="G65" s="26">
-        <f>IF(OR(B65="",E65=""),"",IF(F65&lt;&gt;"","✓ Paid",IF(TODAY()-B65&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B65-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B65)&amp;" day(s)")))</f>
+        <f>IF(OR(B65="",E65=""),"",IF(F65&lt;&gt;"","Paid",IF((TODAY()-B65)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B65-Settings!$C$10)&amp;IF((TODAY()-B65-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B65)&amp;IF((TODAY()-B65)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H65" s="1" t="n"/>
@@ -3592,7 +3603,7 @@
       <c r="E66" s="25" t="n"/>
       <c r="F66" s="23" t="n"/>
       <c r="G66" s="26">
-        <f>IF(OR(B66="",E66=""),"",IF(F66&lt;&gt;"","✓ Paid",IF(TODAY()-B66&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B66-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B66)&amp;" day(s)")))</f>
+        <f>IF(OR(B66="",E66=""),"",IF(F66&lt;&gt;"","Paid",IF((TODAY()-B66)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B66-Settings!$C$10)&amp;IF((TODAY()-B66-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B66)&amp;IF((TODAY()-B66)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H66" s="1" t="n"/>
@@ -3605,7 +3616,7 @@
       <c r="E67" s="25" t="n"/>
       <c r="F67" s="23" t="n"/>
       <c r="G67" s="26">
-        <f>IF(OR(B67="",E67=""),"",IF(F67&lt;&gt;"","✓ Paid",IF(TODAY()-B67&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B67-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B67)&amp;" day(s)")))</f>
+        <f>IF(OR(B67="",E67=""),"",IF(F67&lt;&gt;"","Paid",IF((TODAY()-B67)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B67-Settings!$C$10)&amp;IF((TODAY()-B67-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B67)&amp;IF((TODAY()-B67)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H67" s="1" t="n"/>
@@ -3618,7 +3629,7 @@
       <c r="E68" s="25" t="n"/>
       <c r="F68" s="23" t="n"/>
       <c r="G68" s="26">
-        <f>IF(OR(B68="",E68=""),"",IF(F68&lt;&gt;"","✓ Paid",IF(TODAY()-B68&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B68-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B68)&amp;" day(s)")))</f>
+        <f>IF(OR(B68="",E68=""),"",IF(F68&lt;&gt;"","Paid",IF((TODAY()-B68)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B68-Settings!$C$10)&amp;IF((TODAY()-B68-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B68)&amp;IF((TODAY()-B68)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H68" s="1" t="n"/>
@@ -3631,7 +3642,7 @@
       <c r="E69" s="25" t="n"/>
       <c r="F69" s="23" t="n"/>
       <c r="G69" s="26">
-        <f>IF(OR(B69="",E69=""),"",IF(F69&lt;&gt;"","✓ Paid",IF(TODAY()-B69&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B69-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B69)&amp;" day(s)")))</f>
+        <f>IF(OR(B69="",E69=""),"",IF(F69&lt;&gt;"","Paid",IF((TODAY()-B69)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B69-Settings!$C$10)&amp;IF((TODAY()-B69-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B69)&amp;IF((TODAY()-B69)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H69" s="1" t="n"/>
@@ -3644,7 +3655,7 @@
       <c r="E70" s="25" t="n"/>
       <c r="F70" s="23" t="n"/>
       <c r="G70" s="26">
-        <f>IF(OR(B70="",E70=""),"",IF(F70&lt;&gt;"","✓ Paid",IF(TODAY()-B70&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B70-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B70)&amp;" day(s)")))</f>
+        <f>IF(OR(B70="",E70=""),"",IF(F70&lt;&gt;"","Paid",IF((TODAY()-B70)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B70-Settings!$C$10)&amp;IF((TODAY()-B70-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B70)&amp;IF((TODAY()-B70)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H70" s="1" t="n"/>
@@ -3657,7 +3668,7 @@
       <c r="E71" s="25" t="n"/>
       <c r="F71" s="23" t="n"/>
       <c r="G71" s="26">
-        <f>IF(OR(B71="",E71=""),"",IF(F71&lt;&gt;"","✓ Paid",IF(TODAY()-B71&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B71-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B71)&amp;" day(s)")))</f>
+        <f>IF(OR(B71="",E71=""),"",IF(F71&lt;&gt;"","Paid",IF((TODAY()-B71)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B71-Settings!$C$10)&amp;IF((TODAY()-B71-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B71)&amp;IF((TODAY()-B71)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H71" s="1" t="n"/>
@@ -3670,7 +3681,7 @@
       <c r="E72" s="25" t="n"/>
       <c r="F72" s="23" t="n"/>
       <c r="G72" s="26">
-        <f>IF(OR(B72="",E72=""),"",IF(F72&lt;&gt;"","✓ Paid",IF(TODAY()-B72&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B72-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B72)&amp;" day(s)")))</f>
+        <f>IF(OR(B72="",E72=""),"",IF(F72&lt;&gt;"","Paid",IF((TODAY()-B72)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B72-Settings!$C$10)&amp;IF((TODAY()-B72-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B72)&amp;IF((TODAY()-B72)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H72" s="1" t="n"/>
@@ -3683,7 +3694,7 @@
       <c r="E73" s="25" t="n"/>
       <c r="F73" s="23" t="n"/>
       <c r="G73" s="26">
-        <f>IF(OR(B73="",E73=""),"",IF(F73&lt;&gt;"","✓ Paid",IF(TODAY()-B73&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B73-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B73)&amp;" day(s)")))</f>
+        <f>IF(OR(B73="",E73=""),"",IF(F73&lt;&gt;"","Paid",IF((TODAY()-B73)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B73-Settings!$C$10)&amp;IF((TODAY()-B73-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B73)&amp;IF((TODAY()-B73)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H73" s="1" t="n"/>
@@ -3696,7 +3707,7 @@
       <c r="E74" s="25" t="n"/>
       <c r="F74" s="23" t="n"/>
       <c r="G74" s="26">
-        <f>IF(OR(B74="",E74=""),"",IF(F74&lt;&gt;"","✓ Paid",IF(TODAY()-B74&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B74-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B74)&amp;" day(s)")))</f>
+        <f>IF(OR(B74="",E74=""),"",IF(F74&lt;&gt;"","Paid",IF((TODAY()-B74)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B74-Settings!$C$10)&amp;IF((TODAY()-B74-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B74)&amp;IF((TODAY()-B74)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H74" s="1" t="n"/>
@@ -3709,7 +3720,7 @@
       <c r="E75" s="25" t="n"/>
       <c r="F75" s="23" t="n"/>
       <c r="G75" s="26">
-        <f>IF(OR(B75="",E75=""),"",IF(F75&lt;&gt;"","✓ Paid",IF(TODAY()-B75&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B75-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B75)&amp;" day(s)")))</f>
+        <f>IF(OR(B75="",E75=""),"",IF(F75&lt;&gt;"","Paid",IF((TODAY()-B75)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B75-Settings!$C$10)&amp;IF((TODAY()-B75-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B75)&amp;IF((TODAY()-B75)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H75" s="1" t="n"/>
@@ -3722,7 +3733,7 @@
       <c r="E76" s="25" t="n"/>
       <c r="F76" s="23" t="n"/>
       <c r="G76" s="26">
-        <f>IF(OR(B76="",E76=""),"",IF(F76&lt;&gt;"","✓ Paid",IF(TODAY()-B76&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B76-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B76)&amp;" day(s)")))</f>
+        <f>IF(OR(B76="",E76=""),"",IF(F76&lt;&gt;"","Paid",IF((TODAY()-B76)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B76-Settings!$C$10)&amp;IF((TODAY()-B76-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B76)&amp;IF((TODAY()-B76)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H76" s="1" t="n"/>
@@ -3735,7 +3746,7 @@
       <c r="E77" s="25" t="n"/>
       <c r="F77" s="23" t="n"/>
       <c r="G77" s="26">
-        <f>IF(OR(B77="",E77=""),"",IF(F77&lt;&gt;"","✓ Paid",IF(TODAY()-B77&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B77-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B77)&amp;" day(s)")))</f>
+        <f>IF(OR(B77="",E77=""),"",IF(F77&lt;&gt;"","Paid",IF((TODAY()-B77)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B77-Settings!$C$10)&amp;IF((TODAY()-B77-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B77)&amp;IF((TODAY()-B77)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H77" s="1" t="n"/>
@@ -3748,7 +3759,7 @@
       <c r="E78" s="25" t="n"/>
       <c r="F78" s="23" t="n"/>
       <c r="G78" s="26">
-        <f>IF(OR(B78="",E78=""),"",IF(F78&lt;&gt;"","✓ Paid",IF(TODAY()-B78&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B78-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B78)&amp;" day(s)")))</f>
+        <f>IF(OR(B78="",E78=""),"",IF(F78&lt;&gt;"","Paid",IF((TODAY()-B78)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B78-Settings!$C$10)&amp;IF((TODAY()-B78-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B78)&amp;IF((TODAY()-B78)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H78" s="1" t="n"/>
@@ -3761,7 +3772,7 @@
       <c r="E79" s="25" t="n"/>
       <c r="F79" s="23" t="n"/>
       <c r="G79" s="26">
-        <f>IF(OR(B79="",E79=""),"",IF(F79&lt;&gt;"","✓ Paid",IF(TODAY()-B79&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B79-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B79)&amp;" day(s)")))</f>
+        <f>IF(OR(B79="",E79=""),"",IF(F79&lt;&gt;"","Paid",IF((TODAY()-B79)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B79-Settings!$C$10)&amp;IF((TODAY()-B79-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B79)&amp;IF((TODAY()-B79)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H79" s="1" t="n"/>
@@ -3774,7 +3785,7 @@
       <c r="E80" s="25" t="n"/>
       <c r="F80" s="23" t="n"/>
       <c r="G80" s="26">
-        <f>IF(OR(B80="",E80=""),"",IF(F80&lt;&gt;"","✓ Paid",IF(TODAY()-B80&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B80-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B80)&amp;" day(s)")))</f>
+        <f>IF(OR(B80="",E80=""),"",IF(F80&lt;&gt;"","Paid",IF((TODAY()-B80)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B80-Settings!$C$10)&amp;IF((TODAY()-B80-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B80)&amp;IF((TODAY()-B80)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H80" s="1" t="n"/>
@@ -3787,7 +3798,7 @@
       <c r="E81" s="25" t="n"/>
       <c r="F81" s="23" t="n"/>
       <c r="G81" s="26">
-        <f>IF(OR(B81="",E81=""),"",IF(F81&lt;&gt;"","✓ Paid",IF(TODAY()-B81&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B81-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B81)&amp;" day(s)")))</f>
+        <f>IF(OR(B81="",E81=""),"",IF(F81&lt;&gt;"","Paid",IF((TODAY()-B81)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B81-Settings!$C$10)&amp;IF((TODAY()-B81-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B81)&amp;IF((TODAY()-B81)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H81" s="1" t="n"/>
@@ -3800,7 +3811,7 @@
       <c r="E82" s="25" t="n"/>
       <c r="F82" s="23" t="n"/>
       <c r="G82" s="26">
-        <f>IF(OR(B82="",E82=""),"",IF(F82&lt;&gt;"","✓ Paid",IF(TODAY()-B82&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B82-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B82)&amp;" day(s)")))</f>
+        <f>IF(OR(B82="",E82=""),"",IF(F82&lt;&gt;"","Paid",IF((TODAY()-B82)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B82-Settings!$C$10)&amp;IF((TODAY()-B82-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B82)&amp;IF((TODAY()-B82)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H82" s="1" t="n"/>
@@ -3813,7 +3824,7 @@
       <c r="E83" s="25" t="n"/>
       <c r="F83" s="23" t="n"/>
       <c r="G83" s="26">
-        <f>IF(OR(B83="",E83=""),"",IF(F83&lt;&gt;"","✓ Paid",IF(TODAY()-B83&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B83-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B83)&amp;" day(s)")))</f>
+        <f>IF(OR(B83="",E83=""),"",IF(F83&lt;&gt;"","Paid",IF((TODAY()-B83)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B83-Settings!$C$10)&amp;IF((TODAY()-B83-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B83)&amp;IF((TODAY()-B83)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H83" s="1" t="n"/>
@@ -3826,7 +3837,7 @@
       <c r="E84" s="25" t="n"/>
       <c r="F84" s="23" t="n"/>
       <c r="G84" s="26">
-        <f>IF(OR(B84="",E84=""),"",IF(F84&lt;&gt;"","✓ Paid",IF(TODAY()-B84&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B84-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B84)&amp;" day(s)")))</f>
+        <f>IF(OR(B84="",E84=""),"",IF(F84&lt;&gt;"","Paid",IF((TODAY()-B84)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B84-Settings!$C$10)&amp;IF((TODAY()-B84-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B84)&amp;IF((TODAY()-B84)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H84" s="1" t="n"/>
@@ -3839,7 +3850,7 @@
       <c r="E85" s="25" t="n"/>
       <c r="F85" s="23" t="n"/>
       <c r="G85" s="26">
-        <f>IF(OR(B85="",E85=""),"",IF(F85&lt;&gt;"","✓ Paid",IF(TODAY()-B85&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B85-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B85)&amp;" day(s)")))</f>
+        <f>IF(OR(B85="",E85=""),"",IF(F85&lt;&gt;"","Paid",IF((TODAY()-B85)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B85-Settings!$C$10)&amp;IF((TODAY()-B85-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B85)&amp;IF((TODAY()-B85)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H85" s="1" t="n"/>
@@ -3852,7 +3863,7 @@
       <c r="E86" s="25" t="n"/>
       <c r="F86" s="23" t="n"/>
       <c r="G86" s="26">
-        <f>IF(OR(B86="",E86=""),"",IF(F86&lt;&gt;"","✓ Paid",IF(TODAY()-B86&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B86-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B86)&amp;" day(s)")))</f>
+        <f>IF(OR(B86="",E86=""),"",IF(F86&lt;&gt;"","Paid",IF((TODAY()-B86)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B86-Settings!$C$10)&amp;IF((TODAY()-B86-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B86)&amp;IF((TODAY()-B86)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H86" s="1" t="n"/>
@@ -3865,7 +3876,7 @@
       <c r="E87" s="25" t="n"/>
       <c r="F87" s="23" t="n"/>
       <c r="G87" s="26">
-        <f>IF(OR(B87="",E87=""),"",IF(F87&lt;&gt;"","✓ Paid",IF(TODAY()-B87&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B87-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B87)&amp;" day(s)")))</f>
+        <f>IF(OR(B87="",E87=""),"",IF(F87&lt;&gt;"","Paid",IF((TODAY()-B87)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B87-Settings!$C$10)&amp;IF((TODAY()-B87-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B87)&amp;IF((TODAY()-B87)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H87" s="1" t="n"/>
@@ -3878,7 +3889,7 @@
       <c r="E88" s="25" t="n"/>
       <c r="F88" s="23" t="n"/>
       <c r="G88" s="26">
-        <f>IF(OR(B88="",E88=""),"",IF(F88&lt;&gt;"","✓ Paid",IF(TODAY()-B88&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B88-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B88)&amp;" day(s)")))</f>
+        <f>IF(OR(B88="",E88=""),"",IF(F88&lt;&gt;"","Paid",IF((TODAY()-B88)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B88-Settings!$C$10)&amp;IF((TODAY()-B88-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B88)&amp;IF((TODAY()-B88)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H88" s="1" t="n"/>
@@ -3891,7 +3902,7 @@
       <c r="E89" s="25" t="n"/>
       <c r="F89" s="23" t="n"/>
       <c r="G89" s="26">
-        <f>IF(OR(B89="",E89=""),"",IF(F89&lt;&gt;"","✓ Paid",IF(TODAY()-B89&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B89-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B89)&amp;" day(s)")))</f>
+        <f>IF(OR(B89="",E89=""),"",IF(F89&lt;&gt;"","Paid",IF((TODAY()-B89)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B89-Settings!$C$10)&amp;IF((TODAY()-B89-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B89)&amp;IF((TODAY()-B89)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H89" s="1" t="n"/>
@@ -3904,7 +3915,7 @@
       <c r="E90" s="25" t="n"/>
       <c r="F90" s="23" t="n"/>
       <c r="G90" s="26">
-        <f>IF(OR(B90="",E90=""),"",IF(F90&lt;&gt;"","✓ Paid",IF(TODAY()-B90&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B90-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B90)&amp;" day(s)")))</f>
+        <f>IF(OR(B90="",E90=""),"",IF(F90&lt;&gt;"","Paid",IF((TODAY()-B90)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B90-Settings!$C$10)&amp;IF((TODAY()-B90-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B90)&amp;IF((TODAY()-B90)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H90" s="1" t="n"/>
@@ -3917,7 +3928,7 @@
       <c r="E91" s="25" t="n"/>
       <c r="F91" s="23" t="n"/>
       <c r="G91" s="26">
-        <f>IF(OR(B91="",E91=""),"",IF(F91&lt;&gt;"","✓ Paid",IF(TODAY()-B91&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B91-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B91)&amp;" day(s)")))</f>
+        <f>IF(OR(B91="",E91=""),"",IF(F91&lt;&gt;"","Paid",IF((TODAY()-B91)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B91-Settings!$C$10)&amp;IF((TODAY()-B91-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B91)&amp;IF((TODAY()-B91)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H91" s="1" t="n"/>
@@ -3930,7 +3941,7 @@
       <c r="E92" s="25" t="n"/>
       <c r="F92" s="23" t="n"/>
       <c r="G92" s="26">
-        <f>IF(OR(B92="",E92=""),"",IF(F92&lt;&gt;"","✓ Paid",IF(TODAY()-B92&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B92-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B92)&amp;" day(s)")))</f>
+        <f>IF(OR(B92="",E92=""),"",IF(F92&lt;&gt;"","Paid",IF((TODAY()-B92)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B92-Settings!$C$10)&amp;IF((TODAY()-B92-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B92)&amp;IF((TODAY()-B92)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H92" s="1" t="n"/>
@@ -3943,7 +3954,7 @@
       <c r="E93" s="25" t="n"/>
       <c r="F93" s="23" t="n"/>
       <c r="G93" s="26">
-        <f>IF(OR(B93="",E93=""),"",IF(F93&lt;&gt;"","✓ Paid",IF(TODAY()-B93&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B93-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B93)&amp;" day(s)")))</f>
+        <f>IF(OR(B93="",E93=""),"",IF(F93&lt;&gt;"","Paid",IF((TODAY()-B93)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B93-Settings!$C$10)&amp;IF((TODAY()-B93-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B93)&amp;IF((TODAY()-B93)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H93" s="1" t="n"/>
@@ -3956,7 +3967,7 @@
       <c r="E94" s="25" t="n"/>
       <c r="F94" s="23" t="n"/>
       <c r="G94" s="26">
-        <f>IF(OR(B94="",E94=""),"",IF(F94&lt;&gt;"","✓ Paid",IF(TODAY()-B94&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B94-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B94)&amp;" day(s)")))</f>
+        <f>IF(OR(B94="",E94=""),"",IF(F94&lt;&gt;"","Paid",IF((TODAY()-B94)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B94-Settings!$C$10)&amp;IF((TODAY()-B94-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B94)&amp;IF((TODAY()-B94)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H94" s="1" t="n"/>
@@ -3969,7 +3980,7 @@
       <c r="E95" s="25" t="n"/>
       <c r="F95" s="23" t="n"/>
       <c r="G95" s="26">
-        <f>IF(OR(B95="",E95=""),"",IF(F95&lt;&gt;"","✓ Paid",IF(TODAY()-B95&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B95-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B95)&amp;" day(s)")))</f>
+        <f>IF(OR(B95="",E95=""),"",IF(F95&lt;&gt;"","Paid",IF((TODAY()-B95)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B95-Settings!$C$10)&amp;IF((TODAY()-B95-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B95)&amp;IF((TODAY()-B95)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H95" s="1" t="n"/>
@@ -3982,7 +3993,7 @@
       <c r="E96" s="25" t="n"/>
       <c r="F96" s="23" t="n"/>
       <c r="G96" s="26">
-        <f>IF(OR(B96="",E96=""),"",IF(F96&lt;&gt;"","✓ Paid",IF(TODAY()-B96&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B96-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B96)&amp;" day(s)")))</f>
+        <f>IF(OR(B96="",E96=""),"",IF(F96&lt;&gt;"","Paid",IF((TODAY()-B96)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B96-Settings!$C$10)&amp;IF((TODAY()-B96-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B96)&amp;IF((TODAY()-B96)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H96" s="1" t="n"/>
@@ -3995,7 +4006,7 @@
       <c r="E97" s="25" t="n"/>
       <c r="F97" s="23" t="n"/>
       <c r="G97" s="26">
-        <f>IF(OR(B97="",E97=""),"",IF(F97&lt;&gt;"","✓ Paid",IF(TODAY()-B97&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B97-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B97)&amp;" day(s)")))</f>
+        <f>IF(OR(B97="",E97=""),"",IF(F97&lt;&gt;"","Paid",IF((TODAY()-B97)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B97-Settings!$C$10)&amp;IF((TODAY()-B97-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B97)&amp;IF((TODAY()-B97)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H97" s="1" t="n"/>
@@ -4008,7 +4019,7 @@
       <c r="E98" s="25" t="n"/>
       <c r="F98" s="23" t="n"/>
       <c r="G98" s="26">
-        <f>IF(OR(B98="",E98=""),"",IF(F98&lt;&gt;"","✓ Paid",IF(TODAY()-B98&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B98-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B98)&amp;" day(s)")))</f>
+        <f>IF(OR(B98="",E98=""),"",IF(F98&lt;&gt;"","Paid",IF((TODAY()-B98)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B98-Settings!$C$10)&amp;IF((TODAY()-B98-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B98)&amp;IF((TODAY()-B98)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H98" s="1" t="n"/>
@@ -4021,7 +4032,7 @@
       <c r="E99" s="25" t="n"/>
       <c r="F99" s="23" t="n"/>
       <c r="G99" s="26">
-        <f>IF(OR(B99="",E99=""),"",IF(F99&lt;&gt;"","✓ Paid",IF(TODAY()-B99&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B99-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B99)&amp;" day(s)")))</f>
+        <f>IF(OR(B99="",E99=""),"",IF(F99&lt;&gt;"","Paid",IF((TODAY()-B99)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B99-Settings!$C$10)&amp;IF((TODAY()-B99-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B99)&amp;IF((TODAY()-B99)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H99" s="1" t="n"/>
@@ -4034,7 +4045,7 @@
       <c r="E100" s="25" t="n"/>
       <c r="F100" s="23" t="n"/>
       <c r="G100" s="26">
-        <f>IF(OR(B100="",E100=""),"",IF(F100&lt;&gt;"","✓ Paid",IF(TODAY()-B100&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B100-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B100)&amp;" day(s)")))</f>
+        <f>IF(OR(B100="",E100=""),"",IF(F100&lt;&gt;"","Paid",IF((TODAY()-B100)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B100-Settings!$C$10)&amp;IF((TODAY()-B100-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B100)&amp;IF((TODAY()-B100)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H100" s="1" t="n"/>
@@ -4047,7 +4058,7 @@
       <c r="E101" s="25" t="n"/>
       <c r="F101" s="23" t="n"/>
       <c r="G101" s="26">
-        <f>IF(OR(B101="",E101=""),"",IF(F101&lt;&gt;"","✓ Paid",IF(TODAY()-B101&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B101-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B101)&amp;" day(s)")))</f>
+        <f>IF(OR(B101="",E101=""),"",IF(F101&lt;&gt;"","Paid",IF((TODAY()-B101)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B101-Settings!$C$10)&amp;IF((TODAY()-B101-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B101)&amp;IF((TODAY()-B101)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H101" s="1" t="n"/>
@@ -4060,7 +4071,7 @@
       <c r="E102" s="25" t="n"/>
       <c r="F102" s="23" t="n"/>
       <c r="G102" s="26">
-        <f>IF(OR(B102="",E102=""),"",IF(F102&lt;&gt;"","✓ Paid",IF(TODAY()-B102&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B102-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B102)&amp;" day(s)")))</f>
+        <f>IF(OR(B102="",E102=""),"",IF(F102&lt;&gt;"","Paid",IF((TODAY()-B102)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B102-Settings!$C$10)&amp;IF((TODAY()-B102-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B102)&amp;IF((TODAY()-B102)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H102" s="1" t="n"/>
@@ -4073,7 +4084,7 @@
       <c r="E103" s="25" t="n"/>
       <c r="F103" s="23" t="n"/>
       <c r="G103" s="26">
-        <f>IF(OR(B103="",E103=""),"",IF(F103&lt;&gt;"","✓ Paid",IF(TODAY()-B103&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B103-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B103)&amp;" day(s)")))</f>
+        <f>IF(OR(B103="",E103=""),"",IF(F103&lt;&gt;"","Paid",IF((TODAY()-B103)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B103-Settings!$C$10)&amp;IF((TODAY()-B103-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B103)&amp;IF((TODAY()-B103)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H103" s="1" t="n"/>
@@ -4086,7 +4097,7 @@
       <c r="E104" s="25" t="n"/>
       <c r="F104" s="23" t="n"/>
       <c r="G104" s="26">
-        <f>IF(OR(B104="",E104=""),"",IF(F104&lt;&gt;"","✓ Paid",IF(TODAY()-B104&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B104-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B104)&amp;" day(s)")))</f>
+        <f>IF(OR(B104="",E104=""),"",IF(F104&lt;&gt;"","Paid",IF((TODAY()-B104)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B104-Settings!$C$10)&amp;IF((TODAY()-B104-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B104)&amp;IF((TODAY()-B104)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H104" s="1" t="n"/>
@@ -4099,7 +4110,7 @@
       <c r="E105" s="25" t="n"/>
       <c r="F105" s="23" t="n"/>
       <c r="G105" s="26">
-        <f>IF(OR(B105="",E105=""),"",IF(F105&lt;&gt;"","✓ Paid",IF(TODAY()-B105&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B105-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B105)&amp;" day(s)")))</f>
+        <f>IF(OR(B105="",E105=""),"",IF(F105&lt;&gt;"","Paid",IF((TODAY()-B105)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B105-Settings!$C$10)&amp;IF((TODAY()-B105-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B105)&amp;IF((TODAY()-B105)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H105" s="1" t="n"/>
@@ -4112,7 +4123,7 @@
       <c r="E106" s="25" t="n"/>
       <c r="F106" s="23" t="n"/>
       <c r="G106" s="26">
-        <f>IF(OR(B106="",E106=""),"",IF(F106&lt;&gt;"","✓ Paid",IF(TODAY()-B106&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B106-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B106)&amp;" day(s)")))</f>
+        <f>IF(OR(B106="",E106=""),"",IF(F106&lt;&gt;"","Paid",IF((TODAY()-B106)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B106-Settings!$C$10)&amp;IF((TODAY()-B106-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B106)&amp;IF((TODAY()-B106)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H106" s="1" t="n"/>
@@ -4125,7 +4136,7 @@
       <c r="E107" s="25" t="n"/>
       <c r="F107" s="23" t="n"/>
       <c r="G107" s="26">
-        <f>IF(OR(B107="",E107=""),"",IF(F107&lt;&gt;"","✓ Paid",IF(TODAY()-B107&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B107-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B107)&amp;" day(s)")))</f>
+        <f>IF(OR(B107="",E107=""),"",IF(F107&lt;&gt;"","Paid",IF((TODAY()-B107)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B107-Settings!$C$10)&amp;IF((TODAY()-B107-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B107)&amp;IF((TODAY()-B107)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H107" s="1" t="n"/>
@@ -4138,7 +4149,7 @@
       <c r="E108" s="25" t="n"/>
       <c r="F108" s="23" t="n"/>
       <c r="G108" s="26">
-        <f>IF(OR(B108="",E108=""),"",IF(F108&lt;&gt;"","✓ Paid",IF(TODAY()-B108&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B108-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B108)&amp;" day(s)")))</f>
+        <f>IF(OR(B108="",E108=""),"",IF(F108&lt;&gt;"","Paid",IF((TODAY()-B108)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B108-Settings!$C$10)&amp;IF((TODAY()-B108-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B108)&amp;IF((TODAY()-B108)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H108" s="1" t="n"/>
@@ -4151,7 +4162,7 @@
       <c r="E109" s="25" t="n"/>
       <c r="F109" s="23" t="n"/>
       <c r="G109" s="26">
-        <f>IF(OR(B109="",E109=""),"",IF(F109&lt;&gt;"","✓ Paid",IF(TODAY()-B109&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B109-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B109)&amp;" day(s)")))</f>
+        <f>IF(OR(B109="",E109=""),"",IF(F109&lt;&gt;"","Paid",IF((TODAY()-B109)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B109-Settings!$C$10)&amp;IF((TODAY()-B109-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B109)&amp;IF((TODAY()-B109)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H109" s="1" t="n"/>
@@ -4164,7 +4175,7 @@
       <c r="E110" s="25" t="n"/>
       <c r="F110" s="23" t="n"/>
       <c r="G110" s="26">
-        <f>IF(OR(B110="",E110=""),"",IF(F110&lt;&gt;"","✓ Paid",IF(TODAY()-B110&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B110-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B110)&amp;" day(s)")))</f>
+        <f>IF(OR(B110="",E110=""),"",IF(F110&lt;&gt;"","Paid",IF((TODAY()-B110)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B110-Settings!$C$10)&amp;IF((TODAY()-B110-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B110)&amp;IF((TODAY()-B110)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H110" s="1" t="n"/>
@@ -4177,7 +4188,7 @@
       <c r="E111" s="25" t="n"/>
       <c r="F111" s="23" t="n"/>
       <c r="G111" s="26">
-        <f>IF(OR(B111="",E111=""),"",IF(F111&lt;&gt;"","✓ Paid",IF(TODAY()-B111&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B111-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B111)&amp;" day(s)")))</f>
+        <f>IF(OR(B111="",E111=""),"",IF(F111&lt;&gt;"","Paid",IF((TODAY()-B111)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B111-Settings!$C$10)&amp;IF((TODAY()-B111-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B111)&amp;IF((TODAY()-B111)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H111" s="1" t="n"/>
@@ -4190,7 +4201,7 @@
       <c r="E112" s="25" t="n"/>
       <c r="F112" s="23" t="n"/>
       <c r="G112" s="26">
-        <f>IF(OR(B112="",E112=""),"",IF(F112&lt;&gt;"","✓ Paid",IF(TODAY()-B112&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B112-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B112)&amp;" day(s)")))</f>
+        <f>IF(OR(B112="",E112=""),"",IF(F112&lt;&gt;"","Paid",IF((TODAY()-B112)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B112-Settings!$C$10)&amp;IF((TODAY()-B112-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B112)&amp;IF((TODAY()-B112)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H112" s="1" t="n"/>
@@ -4203,7 +4214,7 @@
       <c r="E113" s="25" t="n"/>
       <c r="F113" s="23" t="n"/>
       <c r="G113" s="26">
-        <f>IF(OR(B113="",E113=""),"",IF(F113&lt;&gt;"","✓ Paid",IF(TODAY()-B113&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B113-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B113)&amp;" day(s)")))</f>
+        <f>IF(OR(B113="",E113=""),"",IF(F113&lt;&gt;"","Paid",IF((TODAY()-B113)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B113-Settings!$C$10)&amp;IF((TODAY()-B113-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B113)&amp;IF((TODAY()-B113)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H113" s="1" t="n"/>
@@ -4216,7 +4227,7 @@
       <c r="E114" s="25" t="n"/>
       <c r="F114" s="23" t="n"/>
       <c r="G114" s="26">
-        <f>IF(OR(B114="",E114=""),"",IF(F114&lt;&gt;"","✓ Paid",IF(TODAY()-B114&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B114-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B114)&amp;" day(s)")))</f>
+        <f>IF(OR(B114="",E114=""),"",IF(F114&lt;&gt;"","Paid",IF((TODAY()-B114)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B114-Settings!$C$10)&amp;IF((TODAY()-B114-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B114)&amp;IF((TODAY()-B114)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H114" s="1" t="n"/>
@@ -4229,7 +4240,7 @@
       <c r="E115" s="25" t="n"/>
       <c r="F115" s="23" t="n"/>
       <c r="G115" s="26">
-        <f>IF(OR(B115="",E115=""),"",IF(F115&lt;&gt;"","✓ Paid",IF(TODAY()-B115&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B115-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B115)&amp;" day(s)")))</f>
+        <f>IF(OR(B115="",E115=""),"",IF(F115&lt;&gt;"","Paid",IF((TODAY()-B115)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B115-Settings!$C$10)&amp;IF((TODAY()-B115-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B115)&amp;IF((TODAY()-B115)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H115" s="1" t="n"/>
@@ -4242,7 +4253,7 @@
       <c r="E116" s="25" t="n"/>
       <c r="F116" s="23" t="n"/>
       <c r="G116" s="26">
-        <f>IF(OR(B116="",E116=""),"",IF(F116&lt;&gt;"","✓ Paid",IF(TODAY()-B116&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B116-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B116)&amp;" day(s)")))</f>
+        <f>IF(OR(B116="",E116=""),"",IF(F116&lt;&gt;"","Paid",IF((TODAY()-B116)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B116-Settings!$C$10)&amp;IF((TODAY()-B116-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B116)&amp;IF((TODAY()-B116)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H116" s="1" t="n"/>
@@ -4255,7 +4266,7 @@
       <c r="E117" s="25" t="n"/>
       <c r="F117" s="23" t="n"/>
       <c r="G117" s="26">
-        <f>IF(OR(B117="",E117=""),"",IF(F117&lt;&gt;"","✓ Paid",IF(TODAY()-B117&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B117-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B117)&amp;" day(s)")))</f>
+        <f>IF(OR(B117="",E117=""),"",IF(F117&lt;&gt;"","Paid",IF((TODAY()-B117)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B117-Settings!$C$10)&amp;IF((TODAY()-B117-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B117)&amp;IF((TODAY()-B117)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H117" s="1" t="n"/>
@@ -4268,7 +4279,7 @@
       <c r="E118" s="25" t="n"/>
       <c r="F118" s="23" t="n"/>
       <c r="G118" s="26">
-        <f>IF(OR(B118="",E118=""),"",IF(F118&lt;&gt;"","✓ Paid",IF(TODAY()-B118&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B118-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B118)&amp;" day(s)")))</f>
+        <f>IF(OR(B118="",E118=""),"",IF(F118&lt;&gt;"","Paid",IF((TODAY()-B118)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B118-Settings!$C$10)&amp;IF((TODAY()-B118-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B118)&amp;IF((TODAY()-B118)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H118" s="1" t="n"/>
@@ -4281,7 +4292,7 @@
       <c r="E119" s="25" t="n"/>
       <c r="F119" s="23" t="n"/>
       <c r="G119" s="26">
-        <f>IF(OR(B119="",E119=""),"",IF(F119&lt;&gt;"","✓ Paid",IF(TODAY()-B119&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B119-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B119)&amp;" day(s)")))</f>
+        <f>IF(OR(B119="",E119=""),"",IF(F119&lt;&gt;"","Paid",IF((TODAY()-B119)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B119-Settings!$C$10)&amp;IF((TODAY()-B119-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B119)&amp;IF((TODAY()-B119)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H119" s="1" t="n"/>
@@ -4294,7 +4305,7 @@
       <c r="E120" s="25" t="n"/>
       <c r="F120" s="23" t="n"/>
       <c r="G120" s="26">
-        <f>IF(OR(B120="",E120=""),"",IF(F120&lt;&gt;"","✓ Paid",IF(TODAY()-B120&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B120-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B120)&amp;" day(s)")))</f>
+        <f>IF(OR(B120="",E120=""),"",IF(F120&lt;&gt;"","Paid",IF((TODAY()-B120)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B120-Settings!$C$10)&amp;IF((TODAY()-B120-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B120)&amp;IF((TODAY()-B120)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H120" s="1" t="n"/>
@@ -4307,7 +4318,7 @@
       <c r="E121" s="25" t="n"/>
       <c r="F121" s="23" t="n"/>
       <c r="G121" s="26">
-        <f>IF(OR(B121="",E121=""),"",IF(F121&lt;&gt;"","✓ Paid",IF(TODAY()-B121&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B121-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B121)&amp;" day(s)")))</f>
+        <f>IF(OR(B121="",E121=""),"",IF(F121&lt;&gt;"","Paid",IF((TODAY()-B121)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B121-Settings!$C$10)&amp;IF((TODAY()-B121-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B121)&amp;IF((TODAY()-B121)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H121" s="1" t="n"/>
@@ -4320,7 +4331,7 @@
       <c r="E122" s="25" t="n"/>
       <c r="F122" s="23" t="n"/>
       <c r="G122" s="26">
-        <f>IF(OR(B122="",E122=""),"",IF(F122&lt;&gt;"","✓ Paid",IF(TODAY()-B122&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B122-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B122)&amp;" day(s)")))</f>
+        <f>IF(OR(B122="",E122=""),"",IF(F122&lt;&gt;"","Paid",IF((TODAY()-B122)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B122-Settings!$C$10)&amp;IF((TODAY()-B122-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B122)&amp;IF((TODAY()-B122)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H122" s="1" t="n"/>
@@ -4333,7 +4344,7 @@
       <c r="E123" s="25" t="n"/>
       <c r="F123" s="23" t="n"/>
       <c r="G123" s="26">
-        <f>IF(OR(B123="",E123=""),"",IF(F123&lt;&gt;"","✓ Paid",IF(TODAY()-B123&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B123-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B123)&amp;" day(s)")))</f>
+        <f>IF(OR(B123="",E123=""),"",IF(F123&lt;&gt;"","Paid",IF((TODAY()-B123)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B123-Settings!$C$10)&amp;IF((TODAY()-B123-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B123)&amp;IF((TODAY()-B123)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H123" s="1" t="n"/>
@@ -4346,7 +4357,7 @@
       <c r="E124" s="25" t="n"/>
       <c r="F124" s="23" t="n"/>
       <c r="G124" s="26">
-        <f>IF(OR(B124="",E124=""),"",IF(F124&lt;&gt;"","✓ Paid",IF(TODAY()-B124&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B124-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B124)&amp;" day(s)")))</f>
+        <f>IF(OR(B124="",E124=""),"",IF(F124&lt;&gt;"","Paid",IF((TODAY()-B124)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B124-Settings!$C$10)&amp;IF((TODAY()-B124-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B124)&amp;IF((TODAY()-B124)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H124" s="1" t="n"/>
@@ -4359,7 +4370,7 @@
       <c r="E125" s="25" t="n"/>
       <c r="F125" s="23" t="n"/>
       <c r="G125" s="26">
-        <f>IF(OR(B125="",E125=""),"",IF(F125&lt;&gt;"","✓ Paid",IF(TODAY()-B125&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B125-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B125)&amp;" day(s)")))</f>
+        <f>IF(OR(B125="",E125=""),"",IF(F125&lt;&gt;"","Paid",IF((TODAY()-B125)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B125-Settings!$C$10)&amp;IF((TODAY()-B125-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B125)&amp;IF((TODAY()-B125)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H125" s="1" t="n"/>
@@ -4372,7 +4383,7 @@
       <c r="E126" s="25" t="n"/>
       <c r="F126" s="23" t="n"/>
       <c r="G126" s="26">
-        <f>IF(OR(B126="",E126=""),"",IF(F126&lt;&gt;"","✓ Paid",IF(TODAY()-B126&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B126-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B126)&amp;" day(s)")))</f>
+        <f>IF(OR(B126="",E126=""),"",IF(F126&lt;&gt;"","Paid",IF((TODAY()-B126)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B126-Settings!$C$10)&amp;IF((TODAY()-B126-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B126)&amp;IF((TODAY()-B126)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H126" s="1" t="n"/>
@@ -4385,7 +4396,7 @@
       <c r="E127" s="25" t="n"/>
       <c r="F127" s="23" t="n"/>
       <c r="G127" s="26">
-        <f>IF(OR(B127="",E127=""),"",IF(F127&lt;&gt;"","✓ Paid",IF(TODAY()-B127&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B127-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B127)&amp;" day(s)")))</f>
+        <f>IF(OR(B127="",E127=""),"",IF(F127&lt;&gt;"","Paid",IF((TODAY()-B127)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B127-Settings!$C$10)&amp;IF((TODAY()-B127-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B127)&amp;IF((TODAY()-B127)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H127" s="1" t="n"/>
@@ -4398,7 +4409,7 @@
       <c r="E128" s="25" t="n"/>
       <c r="F128" s="23" t="n"/>
       <c r="G128" s="26">
-        <f>IF(OR(B128="",E128=""),"",IF(F128&lt;&gt;"","✓ Paid",IF(TODAY()-B128&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B128-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B128)&amp;" day(s)")))</f>
+        <f>IF(OR(B128="",E128=""),"",IF(F128&lt;&gt;"","Paid",IF((TODAY()-B128)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B128-Settings!$C$10)&amp;IF((TODAY()-B128-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B128)&amp;IF((TODAY()-B128)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H128" s="1" t="n"/>
@@ -4411,7 +4422,7 @@
       <c r="E129" s="25" t="n"/>
       <c r="F129" s="23" t="n"/>
       <c r="G129" s="26">
-        <f>IF(OR(B129="",E129=""),"",IF(F129&lt;&gt;"","✓ Paid",IF(TODAY()-B129&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B129-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B129)&amp;" day(s)")))</f>
+        <f>IF(OR(B129="",E129=""),"",IF(F129&lt;&gt;"","Paid",IF((TODAY()-B129)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B129-Settings!$C$10)&amp;IF((TODAY()-B129-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B129)&amp;IF((TODAY()-B129)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H129" s="1" t="n"/>
@@ -4424,7 +4435,7 @@
       <c r="E130" s="25" t="n"/>
       <c r="F130" s="23" t="n"/>
       <c r="G130" s="26">
-        <f>IF(OR(B130="",E130=""),"",IF(F130&lt;&gt;"","✓ Paid",IF(TODAY()-B130&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B130-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B130)&amp;" day(s)")))</f>
+        <f>IF(OR(B130="",E130=""),"",IF(F130&lt;&gt;"","Paid",IF((TODAY()-B130)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B130-Settings!$C$10)&amp;IF((TODAY()-B130-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B130)&amp;IF((TODAY()-B130)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H130" s="1" t="n"/>
@@ -4437,7 +4448,7 @@
       <c r="E131" s="25" t="n"/>
       <c r="F131" s="23" t="n"/>
       <c r="G131" s="26">
-        <f>IF(OR(B131="",E131=""),"",IF(F131&lt;&gt;"","✓ Paid",IF(TODAY()-B131&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B131-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B131)&amp;" day(s)")))</f>
+        <f>IF(OR(B131="",E131=""),"",IF(F131&lt;&gt;"","Paid",IF((TODAY()-B131)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B131-Settings!$C$10)&amp;IF((TODAY()-B131-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B131)&amp;IF((TODAY()-B131)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H131" s="1" t="n"/>
@@ -4450,7 +4461,7 @@
       <c r="E132" s="25" t="n"/>
       <c r="F132" s="23" t="n"/>
       <c r="G132" s="26">
-        <f>IF(OR(B132="",E132=""),"",IF(F132&lt;&gt;"","✓ Paid",IF(TODAY()-B132&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B132-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B132)&amp;" day(s)")))</f>
+        <f>IF(OR(B132="",E132=""),"",IF(F132&lt;&gt;"","Paid",IF((TODAY()-B132)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B132-Settings!$C$10)&amp;IF((TODAY()-B132-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B132)&amp;IF((TODAY()-B132)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H132" s="1" t="n"/>
@@ -4463,7 +4474,7 @@
       <c r="E133" s="25" t="n"/>
       <c r="F133" s="23" t="n"/>
       <c r="G133" s="26">
-        <f>IF(OR(B133="",E133=""),"",IF(F133&lt;&gt;"","✓ Paid",IF(TODAY()-B133&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B133-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B133)&amp;" day(s)")))</f>
+        <f>IF(OR(B133="",E133=""),"",IF(F133&lt;&gt;"","Paid",IF((TODAY()-B133)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B133-Settings!$C$10)&amp;IF((TODAY()-B133-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B133)&amp;IF((TODAY()-B133)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H133" s="1" t="n"/>
@@ -4476,7 +4487,7 @@
       <c r="E134" s="25" t="n"/>
       <c r="F134" s="23" t="n"/>
       <c r="G134" s="26">
-        <f>IF(OR(B134="",E134=""),"",IF(F134&lt;&gt;"","✓ Paid",IF(TODAY()-B134&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B134-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B134)&amp;" day(s)")))</f>
+        <f>IF(OR(B134="",E134=""),"",IF(F134&lt;&gt;"","Paid",IF((TODAY()-B134)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B134-Settings!$C$10)&amp;IF((TODAY()-B134-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B134)&amp;IF((TODAY()-B134)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H134" s="1" t="n"/>
@@ -4489,7 +4500,7 @@
       <c r="E135" s="25" t="n"/>
       <c r="F135" s="23" t="n"/>
       <c r="G135" s="26">
-        <f>IF(OR(B135="",E135=""),"",IF(F135&lt;&gt;"","✓ Paid",IF(TODAY()-B135&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B135-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B135)&amp;" day(s)")))</f>
+        <f>IF(OR(B135="",E135=""),"",IF(F135&lt;&gt;"","Paid",IF((TODAY()-B135)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B135-Settings!$C$10)&amp;IF((TODAY()-B135-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B135)&amp;IF((TODAY()-B135)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H135" s="1" t="n"/>
@@ -4502,7 +4513,7 @@
       <c r="E136" s="25" t="n"/>
       <c r="F136" s="23" t="n"/>
       <c r="G136" s="26">
-        <f>IF(OR(B136="",E136=""),"",IF(F136&lt;&gt;"","✓ Paid",IF(TODAY()-B136&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B136-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B136)&amp;" day(s)")))</f>
+        <f>IF(OR(B136="",E136=""),"",IF(F136&lt;&gt;"","Paid",IF((TODAY()-B136)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B136-Settings!$C$10)&amp;IF((TODAY()-B136-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B136)&amp;IF((TODAY()-B136)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H136" s="1" t="n"/>
@@ -4515,7 +4526,7 @@
       <c r="E137" s="25" t="n"/>
       <c r="F137" s="23" t="n"/>
       <c r="G137" s="26">
-        <f>IF(OR(B137="",E137=""),"",IF(F137&lt;&gt;"","✓ Paid",IF(TODAY()-B137&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B137-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B137)&amp;" day(s)")))</f>
+        <f>IF(OR(B137="",E137=""),"",IF(F137&lt;&gt;"","Paid",IF((TODAY()-B137)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B137-Settings!$C$10)&amp;IF((TODAY()-B137-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B137)&amp;IF((TODAY()-B137)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H137" s="1" t="n"/>
@@ -4528,7 +4539,7 @@
       <c r="E138" s="25" t="n"/>
       <c r="F138" s="23" t="n"/>
       <c r="G138" s="26">
-        <f>IF(OR(B138="",E138=""),"",IF(F138&lt;&gt;"","✓ Paid",IF(TODAY()-B138&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B138-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B138)&amp;" day(s)")))</f>
+        <f>IF(OR(B138="",E138=""),"",IF(F138&lt;&gt;"","Paid",IF((TODAY()-B138)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B138-Settings!$C$10)&amp;IF((TODAY()-B138-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B138)&amp;IF((TODAY()-B138)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H138" s="1" t="n"/>
@@ -4541,7 +4552,7 @@
       <c r="E139" s="25" t="n"/>
       <c r="F139" s="23" t="n"/>
       <c r="G139" s="26">
-        <f>IF(OR(B139="",E139=""),"",IF(F139&lt;&gt;"","✓ Paid",IF(TODAY()-B139&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B139-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B139)&amp;" day(s)")))</f>
+        <f>IF(OR(B139="",E139=""),"",IF(F139&lt;&gt;"","Paid",IF((TODAY()-B139)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B139-Settings!$C$10)&amp;IF((TODAY()-B139-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B139)&amp;IF((TODAY()-B139)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H139" s="1" t="n"/>
@@ -4554,7 +4565,7 @@
       <c r="E140" s="25" t="n"/>
       <c r="F140" s="23" t="n"/>
       <c r="G140" s="26">
-        <f>IF(OR(B140="",E140=""),"",IF(F140&lt;&gt;"","✓ Paid",IF(TODAY()-B140&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B140-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B140)&amp;" day(s)")))</f>
+        <f>IF(OR(B140="",E140=""),"",IF(F140&lt;&gt;"","Paid",IF((TODAY()-B140)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B140-Settings!$C$10)&amp;IF((TODAY()-B140-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B140)&amp;IF((TODAY()-B140)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H140" s="1" t="n"/>
@@ -4567,7 +4578,7 @@
       <c r="E141" s="25" t="n"/>
       <c r="F141" s="23" t="n"/>
       <c r="G141" s="26">
-        <f>IF(OR(B141="",E141=""),"",IF(F141&lt;&gt;"","✓ Paid",IF(TODAY()-B141&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B141-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B141)&amp;" day(s)")))</f>
+        <f>IF(OR(B141="",E141=""),"",IF(F141&lt;&gt;"","Paid",IF((TODAY()-B141)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B141-Settings!$C$10)&amp;IF((TODAY()-B141-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B141)&amp;IF((TODAY()-B141)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H141" s="1" t="n"/>
@@ -4580,7 +4591,7 @@
       <c r="E142" s="25" t="n"/>
       <c r="F142" s="23" t="n"/>
       <c r="G142" s="26">
-        <f>IF(OR(B142="",E142=""),"",IF(F142&lt;&gt;"","✓ Paid",IF(TODAY()-B142&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B142-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B142)&amp;" day(s)")))</f>
+        <f>IF(OR(B142="",E142=""),"",IF(F142&lt;&gt;"","Paid",IF((TODAY()-B142)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B142-Settings!$C$10)&amp;IF((TODAY()-B142-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B142)&amp;IF((TODAY()-B142)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H142" s="1" t="n"/>
@@ -4593,7 +4604,7 @@
       <c r="E143" s="25" t="n"/>
       <c r="F143" s="23" t="n"/>
       <c r="G143" s="26">
-        <f>IF(OR(B143="",E143=""),"",IF(F143&lt;&gt;"","✓ Paid",IF(TODAY()-B143&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B143-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B143)&amp;" day(s)")))</f>
+        <f>IF(OR(B143="",E143=""),"",IF(F143&lt;&gt;"","Paid",IF((TODAY()-B143)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B143-Settings!$C$10)&amp;IF((TODAY()-B143-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B143)&amp;IF((TODAY()-B143)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H143" s="1" t="n"/>
@@ -4606,7 +4617,7 @@
       <c r="E144" s="25" t="n"/>
       <c r="F144" s="23" t="n"/>
       <c r="G144" s="26">
-        <f>IF(OR(B144="",E144=""),"",IF(F144&lt;&gt;"","✓ Paid",IF(TODAY()-B144&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B144-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B144)&amp;" day(s)")))</f>
+        <f>IF(OR(B144="",E144=""),"",IF(F144&lt;&gt;"","Paid",IF((TODAY()-B144)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B144-Settings!$C$10)&amp;IF((TODAY()-B144-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B144)&amp;IF((TODAY()-B144)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H144" s="1" t="n"/>
@@ -4619,7 +4630,7 @@
       <c r="E145" s="25" t="n"/>
       <c r="F145" s="23" t="n"/>
       <c r="G145" s="26">
-        <f>IF(OR(B145="",E145=""),"",IF(F145&lt;&gt;"","✓ Paid",IF(TODAY()-B145&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B145-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B145)&amp;" day(s)")))</f>
+        <f>IF(OR(B145="",E145=""),"",IF(F145&lt;&gt;"","Paid",IF((TODAY()-B145)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B145-Settings!$C$10)&amp;IF((TODAY()-B145-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B145)&amp;IF((TODAY()-B145)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H145" s="1" t="n"/>
@@ -4632,7 +4643,7 @@
       <c r="E146" s="25" t="n"/>
       <c r="F146" s="23" t="n"/>
       <c r="G146" s="26">
-        <f>IF(OR(B146="",E146=""),"",IF(F146&lt;&gt;"","✓ Paid",IF(TODAY()-B146&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B146-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B146)&amp;" day(s)")))</f>
+        <f>IF(OR(B146="",E146=""),"",IF(F146&lt;&gt;"","Paid",IF((TODAY()-B146)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B146-Settings!$C$10)&amp;IF((TODAY()-B146-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B146)&amp;IF((TODAY()-B146)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H146" s="1" t="n"/>
@@ -4645,7 +4656,7 @@
       <c r="E147" s="25" t="n"/>
       <c r="F147" s="23" t="n"/>
       <c r="G147" s="26">
-        <f>IF(OR(B147="",E147=""),"",IF(F147&lt;&gt;"","✓ Paid",IF(TODAY()-B147&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B147-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B147)&amp;" day(s)")))</f>
+        <f>IF(OR(B147="",E147=""),"",IF(F147&lt;&gt;"","Paid",IF((TODAY()-B147)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B147-Settings!$C$10)&amp;IF((TODAY()-B147-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B147)&amp;IF((TODAY()-B147)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H147" s="1" t="n"/>
@@ -4658,7 +4669,7 @@
       <c r="E148" s="25" t="n"/>
       <c r="F148" s="23" t="n"/>
       <c r="G148" s="26">
-        <f>IF(OR(B148="",E148=""),"",IF(F148&lt;&gt;"","✓ Paid",IF(TODAY()-B148&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B148-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B148)&amp;" day(s)")))</f>
+        <f>IF(OR(B148="",E148=""),"",IF(F148&lt;&gt;"","Paid",IF((TODAY()-B148)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B148-Settings!$C$10)&amp;IF((TODAY()-B148-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B148)&amp;IF((TODAY()-B148)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H148" s="1" t="n"/>
@@ -4671,7 +4682,7 @@
       <c r="E149" s="25" t="n"/>
       <c r="F149" s="23" t="n"/>
       <c r="G149" s="26">
-        <f>IF(OR(B149="",E149=""),"",IF(F149&lt;&gt;"","✓ Paid",IF(TODAY()-B149&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B149-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B149)&amp;" day(s)")))</f>
+        <f>IF(OR(B149="",E149=""),"",IF(F149&lt;&gt;"","Paid",IF((TODAY()-B149)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B149-Settings!$C$10)&amp;IF((TODAY()-B149-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B149)&amp;IF((TODAY()-B149)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H149" s="1" t="n"/>
@@ -4684,7 +4695,7 @@
       <c r="E150" s="25" t="n"/>
       <c r="F150" s="23" t="n"/>
       <c r="G150" s="26">
-        <f>IF(OR(B150="",E150=""),"",IF(F150&lt;&gt;"","✓ Paid",IF(TODAY()-B150&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B150-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B150)&amp;" day(s)")))</f>
+        <f>IF(OR(B150="",E150=""),"",IF(F150&lt;&gt;"","Paid",IF((TODAY()-B150)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B150-Settings!$C$10)&amp;IF((TODAY()-B150-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B150)&amp;IF((TODAY()-B150)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H150" s="1" t="n"/>
@@ -4697,7 +4708,7 @@
       <c r="E151" s="25" t="n"/>
       <c r="F151" s="23" t="n"/>
       <c r="G151" s="26">
-        <f>IF(OR(B151="",E151=""),"",IF(F151&lt;&gt;"","✓ Paid",IF(TODAY()-B151&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B151-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B151)&amp;" day(s)")))</f>
+        <f>IF(OR(B151="",E151=""),"",IF(F151&lt;&gt;"","Paid",IF((TODAY()-B151)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B151-Settings!$C$10)&amp;IF((TODAY()-B151-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B151)&amp;IF((TODAY()-B151)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H151" s="1" t="n"/>
@@ -4710,7 +4721,7 @@
       <c r="E152" s="25" t="n"/>
       <c r="F152" s="23" t="n"/>
       <c r="G152" s="26">
-        <f>IF(OR(B152="",E152=""),"",IF(F152&lt;&gt;"","✓ Paid",IF(TODAY()-B152&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B152-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B152)&amp;" day(s)")))</f>
+        <f>IF(OR(B152="",E152=""),"",IF(F152&lt;&gt;"","Paid",IF((TODAY()-B152)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B152-Settings!$C$10)&amp;IF((TODAY()-B152-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B152)&amp;IF((TODAY()-B152)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H152" s="1" t="n"/>
@@ -4723,7 +4734,7 @@
       <c r="E153" s="25" t="n"/>
       <c r="F153" s="23" t="n"/>
       <c r="G153" s="26">
-        <f>IF(OR(B153="",E153=""),"",IF(F153&lt;&gt;"","✓ Paid",IF(TODAY()-B153&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B153-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B153)&amp;" day(s)")))</f>
+        <f>IF(OR(B153="",E153=""),"",IF(F153&lt;&gt;"","Paid",IF((TODAY()-B153)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B153-Settings!$C$10)&amp;IF((TODAY()-B153-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B153)&amp;IF((TODAY()-B153)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H153" s="1" t="n"/>
@@ -4736,7 +4747,7 @@
       <c r="E154" s="25" t="n"/>
       <c r="F154" s="23" t="n"/>
       <c r="G154" s="26">
-        <f>IF(OR(B154="",E154=""),"",IF(F154&lt;&gt;"","✓ Paid",IF(TODAY()-B154&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B154-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B154)&amp;" day(s)")))</f>
+        <f>IF(OR(B154="",E154=""),"",IF(F154&lt;&gt;"","Paid",IF((TODAY()-B154)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B154-Settings!$C$10)&amp;IF((TODAY()-B154-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B154)&amp;IF((TODAY()-B154)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H154" s="1" t="n"/>
@@ -4749,7 +4760,7 @@
       <c r="E155" s="25" t="n"/>
       <c r="F155" s="23" t="n"/>
       <c r="G155" s="26">
-        <f>IF(OR(B155="",E155=""),"",IF(F155&lt;&gt;"","✓ Paid",IF(TODAY()-B155&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B155-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B155)&amp;" day(s)")))</f>
+        <f>IF(OR(B155="",E155=""),"",IF(F155&lt;&gt;"","Paid",IF((TODAY()-B155)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B155-Settings!$C$10)&amp;IF((TODAY()-B155-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B155)&amp;IF((TODAY()-B155)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H155" s="1" t="n"/>
@@ -4762,7 +4773,7 @@
       <c r="E156" s="25" t="n"/>
       <c r="F156" s="23" t="n"/>
       <c r="G156" s="26">
-        <f>IF(OR(B156="",E156=""),"",IF(F156&lt;&gt;"","✓ Paid",IF(TODAY()-B156&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B156-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B156)&amp;" day(s)")))</f>
+        <f>IF(OR(B156="",E156=""),"",IF(F156&lt;&gt;"","Paid",IF((TODAY()-B156)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B156-Settings!$C$10)&amp;IF((TODAY()-B156-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B156)&amp;IF((TODAY()-B156)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H156" s="1" t="n"/>
@@ -4775,7 +4786,7 @@
       <c r="E157" s="25" t="n"/>
       <c r="F157" s="23" t="n"/>
       <c r="G157" s="26">
-        <f>IF(OR(B157="",E157=""),"",IF(F157&lt;&gt;"","✓ Paid",IF(TODAY()-B157&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B157-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B157)&amp;" day(s)")))</f>
+        <f>IF(OR(B157="",E157=""),"",IF(F157&lt;&gt;"","Paid",IF((TODAY()-B157)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B157-Settings!$C$10)&amp;IF((TODAY()-B157-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B157)&amp;IF((TODAY()-B157)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H157" s="1" t="n"/>
@@ -4788,7 +4799,7 @@
       <c r="E158" s="25" t="n"/>
       <c r="F158" s="23" t="n"/>
       <c r="G158" s="26">
-        <f>IF(OR(B158="",E158=""),"",IF(F158&lt;&gt;"","✓ Paid",IF(TODAY()-B158&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B158-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B158)&amp;" day(s)")))</f>
+        <f>IF(OR(B158="",E158=""),"",IF(F158&lt;&gt;"","Paid",IF((TODAY()-B158)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B158-Settings!$C$10)&amp;IF((TODAY()-B158-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B158)&amp;IF((TODAY()-B158)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H158" s="1" t="n"/>
@@ -4801,7 +4812,7 @@
       <c r="E159" s="25" t="n"/>
       <c r="F159" s="23" t="n"/>
       <c r="G159" s="26">
-        <f>IF(OR(B159="",E159=""),"",IF(F159&lt;&gt;"","✓ Paid",IF(TODAY()-B159&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B159-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B159)&amp;" day(s)")))</f>
+        <f>IF(OR(B159="",E159=""),"",IF(F159&lt;&gt;"","Paid",IF((TODAY()-B159)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B159-Settings!$C$10)&amp;IF((TODAY()-B159-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B159)&amp;IF((TODAY()-B159)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H159" s="1" t="n"/>
@@ -4814,7 +4825,7 @@
       <c r="E160" s="25" t="n"/>
       <c r="F160" s="23" t="n"/>
       <c r="G160" s="26">
-        <f>IF(OR(B160="",E160=""),"",IF(F160&lt;&gt;"","✓ Paid",IF(TODAY()-B160&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B160-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B160)&amp;" day(s)")))</f>
+        <f>IF(OR(B160="",E160=""),"",IF(F160&lt;&gt;"","Paid",IF((TODAY()-B160)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B160-Settings!$C$10)&amp;IF((TODAY()-B160-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B160)&amp;IF((TODAY()-B160)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H160" s="1" t="n"/>
@@ -4827,7 +4838,7 @@
       <c r="E161" s="25" t="n"/>
       <c r="F161" s="23" t="n"/>
       <c r="G161" s="26">
-        <f>IF(OR(B161="",E161=""),"",IF(F161&lt;&gt;"","✓ Paid",IF(TODAY()-B161&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B161-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B161)&amp;" day(s)")))</f>
+        <f>IF(OR(B161="",E161=""),"",IF(F161&lt;&gt;"","Paid",IF((TODAY()-B161)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B161-Settings!$C$10)&amp;IF((TODAY()-B161-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B161)&amp;IF((TODAY()-B161)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H161" s="1" t="n"/>
@@ -4840,7 +4851,7 @@
       <c r="E162" s="25" t="n"/>
       <c r="F162" s="23" t="n"/>
       <c r="G162" s="26">
-        <f>IF(OR(B162="",E162=""),"",IF(F162&lt;&gt;"","✓ Paid",IF(TODAY()-B162&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B162-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B162)&amp;" day(s)")))</f>
+        <f>IF(OR(B162="",E162=""),"",IF(F162&lt;&gt;"","Paid",IF((TODAY()-B162)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B162-Settings!$C$10)&amp;IF((TODAY()-B162-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B162)&amp;IF((TODAY()-B162)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H162" s="1" t="n"/>
@@ -4853,7 +4864,7 @@
       <c r="E163" s="25" t="n"/>
       <c r="F163" s="23" t="n"/>
       <c r="G163" s="26">
-        <f>IF(OR(B163="",E163=""),"",IF(F163&lt;&gt;"","✓ Paid",IF(TODAY()-B163&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B163-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B163)&amp;" day(s)")))</f>
+        <f>IF(OR(B163="",E163=""),"",IF(F163&lt;&gt;"","Paid",IF((TODAY()-B163)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B163-Settings!$C$10)&amp;IF((TODAY()-B163-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B163)&amp;IF((TODAY()-B163)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H163" s="1" t="n"/>
@@ -4866,7 +4877,7 @@
       <c r="E164" s="25" t="n"/>
       <c r="F164" s="23" t="n"/>
       <c r="G164" s="26">
-        <f>IF(OR(B164="",E164=""),"",IF(F164&lt;&gt;"","✓ Paid",IF(TODAY()-B164&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B164-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B164)&amp;" day(s)")))</f>
+        <f>IF(OR(B164="",E164=""),"",IF(F164&lt;&gt;"","Paid",IF((TODAY()-B164)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B164-Settings!$C$10)&amp;IF((TODAY()-B164-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B164)&amp;IF((TODAY()-B164)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H164" s="1" t="n"/>
@@ -4879,7 +4890,7 @@
       <c r="E165" s="25" t="n"/>
       <c r="F165" s="23" t="n"/>
       <c r="G165" s="26">
-        <f>IF(OR(B165="",E165=""),"",IF(F165&lt;&gt;"","✓ Paid",IF(TODAY()-B165&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B165-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B165)&amp;" day(s)")))</f>
+        <f>IF(OR(B165="",E165=""),"",IF(F165&lt;&gt;"","Paid",IF((TODAY()-B165)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B165-Settings!$C$10)&amp;IF((TODAY()-B165-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B165)&amp;IF((TODAY()-B165)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H165" s="1" t="n"/>
@@ -4892,7 +4903,7 @@
       <c r="E166" s="25" t="n"/>
       <c r="F166" s="23" t="n"/>
       <c r="G166" s="26">
-        <f>IF(OR(B166="",E166=""),"",IF(F166&lt;&gt;"","✓ Paid",IF(TODAY()-B166&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B166-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B166)&amp;" day(s)")))</f>
+        <f>IF(OR(B166="",E166=""),"",IF(F166&lt;&gt;"","Paid",IF((TODAY()-B166)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B166-Settings!$C$10)&amp;IF((TODAY()-B166-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B166)&amp;IF((TODAY()-B166)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H166" s="1" t="n"/>
@@ -4905,7 +4916,7 @@
       <c r="E167" s="25" t="n"/>
       <c r="F167" s="23" t="n"/>
       <c r="G167" s="26">
-        <f>IF(OR(B167="",E167=""),"",IF(F167&lt;&gt;"","✓ Paid",IF(TODAY()-B167&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B167-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B167)&amp;" day(s)")))</f>
+        <f>IF(OR(B167="",E167=""),"",IF(F167&lt;&gt;"","Paid",IF((TODAY()-B167)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B167-Settings!$C$10)&amp;IF((TODAY()-B167-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B167)&amp;IF((TODAY()-B167)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H167" s="1" t="n"/>
@@ -4918,7 +4929,7 @@
       <c r="E168" s="25" t="n"/>
       <c r="F168" s="23" t="n"/>
       <c r="G168" s="26">
-        <f>IF(OR(B168="",E168=""),"",IF(F168&lt;&gt;"","✓ Paid",IF(TODAY()-B168&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B168-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B168)&amp;" day(s)")))</f>
+        <f>IF(OR(B168="",E168=""),"",IF(F168&lt;&gt;"","Paid",IF((TODAY()-B168)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B168-Settings!$C$10)&amp;IF((TODAY()-B168-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B168)&amp;IF((TODAY()-B168)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H168" s="1" t="n"/>
@@ -4931,7 +4942,7 @@
       <c r="E169" s="25" t="n"/>
       <c r="F169" s="23" t="n"/>
       <c r="G169" s="26">
-        <f>IF(OR(B169="",E169=""),"",IF(F169&lt;&gt;"","✓ Paid",IF(TODAY()-B169&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B169-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B169)&amp;" day(s)")))</f>
+        <f>IF(OR(B169="",E169=""),"",IF(F169&lt;&gt;"","Paid",IF((TODAY()-B169)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B169-Settings!$C$10)&amp;IF((TODAY()-B169-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B169)&amp;IF((TODAY()-B169)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H169" s="1" t="n"/>
@@ -4944,7 +4955,7 @@
       <c r="E170" s="25" t="n"/>
       <c r="F170" s="23" t="n"/>
       <c r="G170" s="26">
-        <f>IF(OR(B170="",E170=""),"",IF(F170&lt;&gt;"","✓ Paid",IF(TODAY()-B170&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B170-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B170)&amp;" day(s)")))</f>
+        <f>IF(OR(B170="",E170=""),"",IF(F170&lt;&gt;"","Paid",IF((TODAY()-B170)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B170-Settings!$C$10)&amp;IF((TODAY()-B170-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B170)&amp;IF((TODAY()-B170)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H170" s="1" t="n"/>
@@ -4957,7 +4968,7 @@
       <c r="E171" s="25" t="n"/>
       <c r="F171" s="23" t="n"/>
       <c r="G171" s="26">
-        <f>IF(OR(B171="",E171=""),"",IF(F171&lt;&gt;"","✓ Paid",IF(TODAY()-B171&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B171-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B171)&amp;" day(s)")))</f>
+        <f>IF(OR(B171="",E171=""),"",IF(F171&lt;&gt;"","Paid",IF((TODAY()-B171)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B171-Settings!$C$10)&amp;IF((TODAY()-B171-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B171)&amp;IF((TODAY()-B171)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H171" s="1" t="n"/>
@@ -4970,7 +4981,7 @@
       <c r="E172" s="25" t="n"/>
       <c r="F172" s="23" t="n"/>
       <c r="G172" s="26">
-        <f>IF(OR(B172="",E172=""),"",IF(F172&lt;&gt;"","✓ Paid",IF(TODAY()-B172&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B172-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B172)&amp;" day(s)")))</f>
+        <f>IF(OR(B172="",E172=""),"",IF(F172&lt;&gt;"","Paid",IF((TODAY()-B172)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B172-Settings!$C$10)&amp;IF((TODAY()-B172-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B172)&amp;IF((TODAY()-B172)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H172" s="1" t="n"/>
@@ -4983,7 +4994,7 @@
       <c r="E173" s="25" t="n"/>
       <c r="F173" s="23" t="n"/>
       <c r="G173" s="26">
-        <f>IF(OR(B173="",E173=""),"",IF(F173&lt;&gt;"","✓ Paid",IF(TODAY()-B173&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B173-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B173)&amp;" day(s)")))</f>
+        <f>IF(OR(B173="",E173=""),"",IF(F173&lt;&gt;"","Paid",IF((TODAY()-B173)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B173-Settings!$C$10)&amp;IF((TODAY()-B173-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B173)&amp;IF((TODAY()-B173)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H173" s="1" t="n"/>
@@ -4996,7 +5007,7 @@
       <c r="E174" s="25" t="n"/>
       <c r="F174" s="23" t="n"/>
       <c r="G174" s="26">
-        <f>IF(OR(B174="",E174=""),"",IF(F174&lt;&gt;"","✓ Paid",IF(TODAY()-B174&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B174-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B174)&amp;" day(s)")))</f>
+        <f>IF(OR(B174="",E174=""),"",IF(F174&lt;&gt;"","Paid",IF((TODAY()-B174)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B174-Settings!$C$10)&amp;IF((TODAY()-B174-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B174)&amp;IF((TODAY()-B174)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H174" s="1" t="n"/>
@@ -5009,7 +5020,7 @@
       <c r="E175" s="25" t="n"/>
       <c r="F175" s="23" t="n"/>
       <c r="G175" s="26">
-        <f>IF(OR(B175="",E175=""),"",IF(F175&lt;&gt;"","✓ Paid",IF(TODAY()-B175&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B175-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B175)&amp;" day(s)")))</f>
+        <f>IF(OR(B175="",E175=""),"",IF(F175&lt;&gt;"","Paid",IF((TODAY()-B175)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B175-Settings!$C$10)&amp;IF((TODAY()-B175-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B175)&amp;IF((TODAY()-B175)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H175" s="1" t="n"/>
@@ -5022,7 +5033,7 @@
       <c r="E176" s="25" t="n"/>
       <c r="F176" s="23" t="n"/>
       <c r="G176" s="26">
-        <f>IF(OR(B176="",E176=""),"",IF(F176&lt;&gt;"","✓ Paid",IF(TODAY()-B176&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B176-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B176)&amp;" day(s)")))</f>
+        <f>IF(OR(B176="",E176=""),"",IF(F176&lt;&gt;"","Paid",IF((TODAY()-B176)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B176-Settings!$C$10)&amp;IF((TODAY()-B176-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B176)&amp;IF((TODAY()-B176)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H176" s="1" t="n"/>
@@ -5035,7 +5046,7 @@
       <c r="E177" s="25" t="n"/>
       <c r="F177" s="23" t="n"/>
       <c r="G177" s="26">
-        <f>IF(OR(B177="",E177=""),"",IF(F177&lt;&gt;"","✓ Paid",IF(TODAY()-B177&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B177-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B177)&amp;" day(s)")))</f>
+        <f>IF(OR(B177="",E177=""),"",IF(F177&lt;&gt;"","Paid",IF((TODAY()-B177)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B177-Settings!$C$10)&amp;IF((TODAY()-B177-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B177)&amp;IF((TODAY()-B177)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H177" s="1" t="n"/>
@@ -5048,7 +5059,7 @@
       <c r="E178" s="25" t="n"/>
       <c r="F178" s="23" t="n"/>
       <c r="G178" s="26">
-        <f>IF(OR(B178="",E178=""),"",IF(F178&lt;&gt;"","✓ Paid",IF(TODAY()-B178&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B178-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B178)&amp;" day(s)")))</f>
+        <f>IF(OR(B178="",E178=""),"",IF(F178&lt;&gt;"","Paid",IF((TODAY()-B178)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B178-Settings!$C$10)&amp;IF((TODAY()-B178-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B178)&amp;IF((TODAY()-B178)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H178" s="1" t="n"/>
@@ -5061,7 +5072,7 @@
       <c r="E179" s="25" t="n"/>
       <c r="F179" s="23" t="n"/>
       <c r="G179" s="26">
-        <f>IF(OR(B179="",E179=""),"",IF(F179&lt;&gt;"","✓ Paid",IF(TODAY()-B179&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B179-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B179)&amp;" day(s)")))</f>
+        <f>IF(OR(B179="",E179=""),"",IF(F179&lt;&gt;"","Paid",IF((TODAY()-B179)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B179-Settings!$C$10)&amp;IF((TODAY()-B179-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B179)&amp;IF((TODAY()-B179)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H179" s="1" t="n"/>
@@ -5074,7 +5085,7 @@
       <c r="E180" s="25" t="n"/>
       <c r="F180" s="23" t="n"/>
       <c r="G180" s="26">
-        <f>IF(OR(B180="",E180=""),"",IF(F180&lt;&gt;"","✓ Paid",IF(TODAY()-B180&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B180-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B180)&amp;" day(s)")))</f>
+        <f>IF(OR(B180="",E180=""),"",IF(F180&lt;&gt;"","Paid",IF((TODAY()-B180)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B180-Settings!$C$10)&amp;IF((TODAY()-B180-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B180)&amp;IF((TODAY()-B180)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H180" s="1" t="n"/>
@@ -5087,7 +5098,7 @@
       <c r="E181" s="25" t="n"/>
       <c r="F181" s="23" t="n"/>
       <c r="G181" s="26">
-        <f>IF(OR(B181="",E181=""),"",IF(F181&lt;&gt;"","✓ Paid",IF(TODAY()-B181&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B181-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B181)&amp;" day(s)")))</f>
+        <f>IF(OR(B181="",E181=""),"",IF(F181&lt;&gt;"","Paid",IF((TODAY()-B181)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B181-Settings!$C$10)&amp;IF((TODAY()-B181-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B181)&amp;IF((TODAY()-B181)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H181" s="1" t="n"/>
@@ -5100,7 +5111,7 @@
       <c r="E182" s="25" t="n"/>
       <c r="F182" s="23" t="n"/>
       <c r="G182" s="26">
-        <f>IF(OR(B182="",E182=""),"",IF(F182&lt;&gt;"","✓ Paid",IF(TODAY()-B182&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B182-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B182)&amp;" day(s)")))</f>
+        <f>IF(OR(B182="",E182=""),"",IF(F182&lt;&gt;"","Paid",IF((TODAY()-B182)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B182-Settings!$C$10)&amp;IF((TODAY()-B182-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B182)&amp;IF((TODAY()-B182)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H182" s="1" t="n"/>
@@ -5113,7 +5124,7 @@
       <c r="E183" s="25" t="n"/>
       <c r="F183" s="23" t="n"/>
       <c r="G183" s="26">
-        <f>IF(OR(B183="",E183=""),"",IF(F183&lt;&gt;"","✓ Paid",IF(TODAY()-B183&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B183-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B183)&amp;" day(s)")))</f>
+        <f>IF(OR(B183="",E183=""),"",IF(F183&lt;&gt;"","Paid",IF((TODAY()-B183)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B183-Settings!$C$10)&amp;IF((TODAY()-B183-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B183)&amp;IF((TODAY()-B183)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H183" s="1" t="n"/>
@@ -5126,7 +5137,7 @@
       <c r="E184" s="25" t="n"/>
       <c r="F184" s="23" t="n"/>
       <c r="G184" s="26">
-        <f>IF(OR(B184="",E184=""),"",IF(F184&lt;&gt;"","✓ Paid",IF(TODAY()-B184&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B184-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B184)&amp;" day(s)")))</f>
+        <f>IF(OR(B184="",E184=""),"",IF(F184&lt;&gt;"","Paid",IF((TODAY()-B184)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B184-Settings!$C$10)&amp;IF((TODAY()-B184-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B184)&amp;IF((TODAY()-B184)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H184" s="1" t="n"/>
@@ -5139,7 +5150,7 @@
       <c r="E185" s="25" t="n"/>
       <c r="F185" s="23" t="n"/>
       <c r="G185" s="26">
-        <f>IF(OR(B185="",E185=""),"",IF(F185&lt;&gt;"","✓ Paid",IF(TODAY()-B185&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B185-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B185)&amp;" day(s)")))</f>
+        <f>IF(OR(B185="",E185=""),"",IF(F185&lt;&gt;"","Paid",IF((TODAY()-B185)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B185-Settings!$C$10)&amp;IF((TODAY()-B185-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B185)&amp;IF((TODAY()-B185)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H185" s="1" t="n"/>
@@ -5152,7 +5163,7 @@
       <c r="E186" s="25" t="n"/>
       <c r="F186" s="23" t="n"/>
       <c r="G186" s="26">
-        <f>IF(OR(B186="",E186=""),"",IF(F186&lt;&gt;"","✓ Paid",IF(TODAY()-B186&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B186-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B186)&amp;" day(s)")))</f>
+        <f>IF(OR(B186="",E186=""),"",IF(F186&lt;&gt;"","Paid",IF((TODAY()-B186)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B186-Settings!$C$10)&amp;IF((TODAY()-B186-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B186)&amp;IF((TODAY()-B186)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H186" s="1" t="n"/>
@@ -5165,7 +5176,7 @@
       <c r="E187" s="25" t="n"/>
       <c r="F187" s="23" t="n"/>
       <c r="G187" s="26">
-        <f>IF(OR(B187="",E187=""),"",IF(F187&lt;&gt;"","✓ Paid",IF(TODAY()-B187&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B187-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B187)&amp;" day(s)")))</f>
+        <f>IF(OR(B187="",E187=""),"",IF(F187&lt;&gt;"","Paid",IF((TODAY()-B187)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B187-Settings!$C$10)&amp;IF((TODAY()-B187-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B187)&amp;IF((TODAY()-B187)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H187" s="1" t="n"/>
@@ -5178,7 +5189,7 @@
       <c r="E188" s="25" t="n"/>
       <c r="F188" s="23" t="n"/>
       <c r="G188" s="26">
-        <f>IF(OR(B188="",E188=""),"",IF(F188&lt;&gt;"","✓ Paid",IF(TODAY()-B188&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B188-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B188)&amp;" day(s)")))</f>
+        <f>IF(OR(B188="",E188=""),"",IF(F188&lt;&gt;"","Paid",IF((TODAY()-B188)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B188-Settings!$C$10)&amp;IF((TODAY()-B188-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B188)&amp;IF((TODAY()-B188)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H188" s="1" t="n"/>
@@ -5191,7 +5202,7 @@
       <c r="E189" s="25" t="n"/>
       <c r="F189" s="23" t="n"/>
       <c r="G189" s="26">
-        <f>IF(OR(B189="",E189=""),"",IF(F189&lt;&gt;"","✓ Paid",IF(TODAY()-B189&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B189-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B189)&amp;" day(s)")))</f>
+        <f>IF(OR(B189="",E189=""),"",IF(F189&lt;&gt;"","Paid",IF((TODAY()-B189)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B189-Settings!$C$10)&amp;IF((TODAY()-B189-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B189)&amp;IF((TODAY()-B189)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H189" s="1" t="n"/>
@@ -5204,7 +5215,7 @@
       <c r="E190" s="25" t="n"/>
       <c r="F190" s="23" t="n"/>
       <c r="G190" s="26">
-        <f>IF(OR(B190="",E190=""),"",IF(F190&lt;&gt;"","✓ Paid",IF(TODAY()-B190&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B190-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B190)&amp;" day(s)")))</f>
+        <f>IF(OR(B190="",E190=""),"",IF(F190&lt;&gt;"","Paid",IF((TODAY()-B190)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B190-Settings!$C$10)&amp;IF((TODAY()-B190-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B190)&amp;IF((TODAY()-B190)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H190" s="1" t="n"/>
@@ -5217,7 +5228,7 @@
       <c r="E191" s="25" t="n"/>
       <c r="F191" s="23" t="n"/>
       <c r="G191" s="26">
-        <f>IF(OR(B191="",E191=""),"",IF(F191&lt;&gt;"","✓ Paid",IF(TODAY()-B191&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B191-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B191)&amp;" day(s)")))</f>
+        <f>IF(OR(B191="",E191=""),"",IF(F191&lt;&gt;"","Paid",IF((TODAY()-B191)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B191-Settings!$C$10)&amp;IF((TODAY()-B191-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B191)&amp;IF((TODAY()-B191)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H191" s="1" t="n"/>
@@ -5230,7 +5241,7 @@
       <c r="E192" s="25" t="n"/>
       <c r="F192" s="23" t="n"/>
       <c r="G192" s="26">
-        <f>IF(OR(B192="",E192=""),"",IF(F192&lt;&gt;"","✓ Paid",IF(TODAY()-B192&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B192-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B192)&amp;" day(s)")))</f>
+        <f>IF(OR(B192="",E192=""),"",IF(F192&lt;&gt;"","Paid",IF((TODAY()-B192)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B192-Settings!$C$10)&amp;IF((TODAY()-B192-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B192)&amp;IF((TODAY()-B192)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H192" s="1" t="n"/>
@@ -5243,7 +5254,7 @@
       <c r="E193" s="25" t="n"/>
       <c r="F193" s="23" t="n"/>
       <c r="G193" s="26">
-        <f>IF(OR(B193="",E193=""),"",IF(F193&lt;&gt;"","✓ Paid",IF(TODAY()-B193&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B193-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B193)&amp;" day(s)")))</f>
+        <f>IF(OR(B193="",E193=""),"",IF(F193&lt;&gt;"","Paid",IF((TODAY()-B193)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B193-Settings!$C$10)&amp;IF((TODAY()-B193-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B193)&amp;IF((TODAY()-B193)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H193" s="1" t="n"/>
@@ -5256,7 +5267,7 @@
       <c r="E194" s="25" t="n"/>
       <c r="F194" s="23" t="n"/>
       <c r="G194" s="26">
-        <f>IF(OR(B194="",E194=""),"",IF(F194&lt;&gt;"","✓ Paid",IF(TODAY()-B194&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B194-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B194)&amp;" day(s)")))</f>
+        <f>IF(OR(B194="",E194=""),"",IF(F194&lt;&gt;"","Paid",IF((TODAY()-B194)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B194-Settings!$C$10)&amp;IF((TODAY()-B194-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B194)&amp;IF((TODAY()-B194)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H194" s="1" t="n"/>
@@ -5269,7 +5280,7 @@
       <c r="E195" s="25" t="n"/>
       <c r="F195" s="23" t="n"/>
       <c r="G195" s="26">
-        <f>IF(OR(B195="",E195=""),"",IF(F195&lt;&gt;"","✓ Paid",IF(TODAY()-B195&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B195-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B195)&amp;" day(s)")))</f>
+        <f>IF(OR(B195="",E195=""),"",IF(F195&lt;&gt;"","Paid",IF((TODAY()-B195)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B195-Settings!$C$10)&amp;IF((TODAY()-B195-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B195)&amp;IF((TODAY()-B195)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H195" s="1" t="n"/>
@@ -5282,7 +5293,7 @@
       <c r="E196" s="25" t="n"/>
       <c r="F196" s="23" t="n"/>
       <c r="G196" s="26">
-        <f>IF(OR(B196="",E196=""),"",IF(F196&lt;&gt;"","✓ Paid",IF(TODAY()-B196&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B196-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B196)&amp;" day(s)")))</f>
+        <f>IF(OR(B196="",E196=""),"",IF(F196&lt;&gt;"","Paid",IF((TODAY()-B196)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B196-Settings!$C$10)&amp;IF((TODAY()-B196-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B196)&amp;IF((TODAY()-B196)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H196" s="1" t="n"/>
@@ -5295,7 +5306,7 @@
       <c r="E197" s="25" t="n"/>
       <c r="F197" s="23" t="n"/>
       <c r="G197" s="26">
-        <f>IF(OR(B197="",E197=""),"",IF(F197&lt;&gt;"","✓ Paid",IF(TODAY()-B197&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B197-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B197)&amp;" day(s)")))</f>
+        <f>IF(OR(B197="",E197=""),"",IF(F197&lt;&gt;"","Paid",IF((TODAY()-B197)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B197-Settings!$C$10)&amp;IF((TODAY()-B197-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B197)&amp;IF((TODAY()-B197)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H197" s="1" t="n"/>
@@ -5308,7 +5319,7 @@
       <c r="E198" s="25" t="n"/>
       <c r="F198" s="23" t="n"/>
       <c r="G198" s="26">
-        <f>IF(OR(B198="",E198=""),"",IF(F198&lt;&gt;"","✓ Paid",IF(TODAY()-B198&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B198-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B198)&amp;" day(s)")))</f>
+        <f>IF(OR(B198="",E198=""),"",IF(F198&lt;&gt;"","Paid",IF((TODAY()-B198)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B198-Settings!$C$10)&amp;IF((TODAY()-B198-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B198)&amp;IF((TODAY()-B198)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H198" s="1" t="n"/>
@@ -5321,7 +5332,7 @@
       <c r="E199" s="25" t="n"/>
       <c r="F199" s="23" t="n"/>
       <c r="G199" s="26">
-        <f>IF(OR(B199="",E199=""),"",IF(F199&lt;&gt;"","✓ Paid",IF(TODAY()-B199&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B199-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B199)&amp;" day(s)")))</f>
+        <f>IF(OR(B199="",E199=""),"",IF(F199&lt;&gt;"","Paid",IF((TODAY()-B199)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B199-Settings!$C$10)&amp;IF((TODAY()-B199-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B199)&amp;IF((TODAY()-B199)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H199" s="1" t="n"/>
@@ -5334,7 +5345,7 @@
       <c r="E200" s="25" t="n"/>
       <c r="F200" s="23" t="n"/>
       <c r="G200" s="26">
-        <f>IF(OR(B200="",E200=""),"",IF(F200&lt;&gt;"","✓ Paid",IF(TODAY()-B200&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B200-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B200)&amp;" day(s)")))</f>
+        <f>IF(OR(B200="",E200=""),"",IF(F200&lt;&gt;"","Paid",IF((TODAY()-B200)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B200-Settings!$C$10)&amp;IF((TODAY()-B200-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B200)&amp;IF((TODAY()-B200)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H200" s="1" t="n"/>
@@ -5347,7 +5358,7 @@
       <c r="E201" s="25" t="n"/>
       <c r="F201" s="23" t="n"/>
       <c r="G201" s="26">
-        <f>IF(OR(B201="",E201=""),"",IF(F201&lt;&gt;"","✓ Paid",IF(TODAY()-B201&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B201-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B201)&amp;" day(s)")))</f>
+        <f>IF(OR(B201="",E201=""),"",IF(F201&lt;&gt;"","Paid",IF((TODAY()-B201)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B201-Settings!$C$10)&amp;IF((TODAY()-B201-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B201)&amp;IF((TODAY()-B201)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H201" s="1" t="n"/>
@@ -5360,7 +5371,7 @@
       <c r="E202" s="25" t="n"/>
       <c r="F202" s="23" t="n"/>
       <c r="G202" s="26">
-        <f>IF(OR(B202="",E202=""),"",IF(F202&lt;&gt;"","✓ Paid",IF(TODAY()-B202&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B202-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B202)&amp;" day(s)")))</f>
+        <f>IF(OR(B202="",E202=""),"",IF(F202&lt;&gt;"","Paid",IF((TODAY()-B202)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B202-Settings!$C$10)&amp;IF((TODAY()-B202-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B202)&amp;IF((TODAY()-B202)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H202" s="1" t="n"/>
@@ -5373,7 +5384,7 @@
       <c r="E203" s="25" t="n"/>
       <c r="F203" s="23" t="n"/>
       <c r="G203" s="26">
-        <f>IF(OR(B203="",E203=""),"",IF(F203&lt;&gt;"","✓ Paid",IF(TODAY()-B203&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B203-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B203)&amp;" day(s)")))</f>
+        <f>IF(OR(B203="",E203=""),"",IF(F203&lt;&gt;"","Paid",IF((TODAY()-B203)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B203-Settings!$C$10)&amp;IF((TODAY()-B203-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B203)&amp;IF((TODAY()-B203)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H203" s="1" t="n"/>
@@ -5386,7 +5397,7 @@
       <c r="E204" s="25" t="n"/>
       <c r="F204" s="23" t="n"/>
       <c r="G204" s="26">
-        <f>IF(OR(B204="",E204=""),"",IF(F204&lt;&gt;"","✓ Paid",IF(TODAY()-B204&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B204-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B204)&amp;" day(s)")))</f>
+        <f>IF(OR(B204="",E204=""),"",IF(F204&lt;&gt;"","Paid",IF((TODAY()-B204)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B204-Settings!$C$10)&amp;IF((TODAY()-B204-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B204)&amp;IF((TODAY()-B204)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H204" s="1" t="n"/>
@@ -5399,7 +5410,7 @@
       <c r="E205" s="25" t="n"/>
       <c r="F205" s="23" t="n"/>
       <c r="G205" s="26">
-        <f>IF(OR(B205="",E205=""),"",IF(F205&lt;&gt;"","✓ Paid",IF(TODAY()-B205&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B205-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B205)&amp;" day(s)")))</f>
+        <f>IF(OR(B205="",E205=""),"",IF(F205&lt;&gt;"","Paid",IF((TODAY()-B205)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B205-Settings!$C$10)&amp;IF((TODAY()-B205-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B205)&amp;IF((TODAY()-B205)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H205" s="1" t="n"/>
@@ -5412,7 +5423,7 @@
       <c r="E206" s="25" t="n"/>
       <c r="F206" s="23" t="n"/>
       <c r="G206" s="26">
-        <f>IF(OR(B206="",E206=""),"",IF(F206&lt;&gt;"","✓ Paid",IF(TODAY()-B206&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B206-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B206)&amp;" day(s)")))</f>
+        <f>IF(OR(B206="",E206=""),"",IF(F206&lt;&gt;"","Paid",IF((TODAY()-B206)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B206-Settings!$C$10)&amp;IF((TODAY()-B206-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B206)&amp;IF((TODAY()-B206)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H206" s="1" t="n"/>
@@ -5425,7 +5436,7 @@
       <c r="E207" s="25" t="n"/>
       <c r="F207" s="23" t="n"/>
       <c r="G207" s="26">
-        <f>IF(OR(B207="",E207=""),"",IF(F207&lt;&gt;"","✓ Paid",IF(TODAY()-B207&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B207-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B207)&amp;" day(s)")))</f>
+        <f>IF(OR(B207="",E207=""),"",IF(F207&lt;&gt;"","Paid",IF((TODAY()-B207)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B207-Settings!$C$10)&amp;IF((TODAY()-B207-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B207)&amp;IF((TODAY()-B207)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H207" s="1" t="n"/>
@@ -5438,7 +5449,7 @@
       <c r="E208" s="25" t="n"/>
       <c r="F208" s="23" t="n"/>
       <c r="G208" s="26">
-        <f>IF(OR(B208="",E208=""),"",IF(F208&lt;&gt;"","✓ Paid",IF(TODAY()-B208&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B208-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B208)&amp;" day(s)")))</f>
+        <f>IF(OR(B208="",E208=""),"",IF(F208&lt;&gt;"","Paid",IF((TODAY()-B208)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B208-Settings!$C$10)&amp;IF((TODAY()-B208-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B208)&amp;IF((TODAY()-B208)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H208" s="1" t="n"/>
@@ -5451,7 +5462,7 @@
       <c r="E209" s="25" t="n"/>
       <c r="F209" s="23" t="n"/>
       <c r="G209" s="26">
-        <f>IF(OR(B209="",E209=""),"",IF(F209&lt;&gt;"","✓ Paid",IF(TODAY()-B209&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B209-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B209)&amp;" day(s)")))</f>
+        <f>IF(OR(B209="",E209=""),"",IF(F209&lt;&gt;"","Paid",IF((TODAY()-B209)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B209-Settings!$C$10)&amp;IF((TODAY()-B209-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B209)&amp;IF((TODAY()-B209)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H209" s="1" t="n"/>
@@ -5464,7 +5475,7 @@
       <c r="E210" s="25" t="n"/>
       <c r="F210" s="23" t="n"/>
       <c r="G210" s="26">
-        <f>IF(OR(B210="",E210=""),"",IF(F210&lt;&gt;"","✓ Paid",IF(TODAY()-B210&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B210-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B210)&amp;" day(s)")))</f>
+        <f>IF(OR(B210="",E210=""),"",IF(F210&lt;&gt;"","Paid",IF((TODAY()-B210)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B210-Settings!$C$10)&amp;IF((TODAY()-B210-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B210)&amp;IF((TODAY()-B210)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H210" s="1" t="n"/>
@@ -5477,7 +5488,7 @@
       <c r="E211" s="25" t="n"/>
       <c r="F211" s="23" t="n"/>
       <c r="G211" s="26">
-        <f>IF(OR(B211="",E211=""),"",IF(F211&lt;&gt;"","✓ Paid",IF(TODAY()-B211&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B211-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B211)&amp;" day(s)")))</f>
+        <f>IF(OR(B211="",E211=""),"",IF(F211&lt;&gt;"","Paid",IF((TODAY()-B211)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B211-Settings!$C$10)&amp;IF((TODAY()-B211-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B211)&amp;IF((TODAY()-B211)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H211" s="1" t="n"/>
@@ -5490,7 +5501,7 @@
       <c r="E212" s="25" t="n"/>
       <c r="F212" s="23" t="n"/>
       <c r="G212" s="26">
-        <f>IF(OR(B212="",E212=""),"",IF(F212&lt;&gt;"","✓ Paid",IF(TODAY()-B212&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B212-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B212)&amp;" day(s)")))</f>
+        <f>IF(OR(B212="",E212=""),"",IF(F212&lt;&gt;"","Paid",IF((TODAY()-B212)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B212-Settings!$C$10)&amp;IF((TODAY()-B212-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B212)&amp;IF((TODAY()-B212)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H212" s="1" t="n"/>
@@ -5503,7 +5514,7 @@
       <c r="E213" s="25" t="n"/>
       <c r="F213" s="23" t="n"/>
       <c r="G213" s="26">
-        <f>IF(OR(B213="",E213=""),"",IF(F213&lt;&gt;"","✓ Paid",IF(TODAY()-B213&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B213-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B213)&amp;" day(s)")))</f>
+        <f>IF(OR(B213="",E213=""),"",IF(F213&lt;&gt;"","Paid",IF((TODAY()-B213)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B213-Settings!$C$10)&amp;IF((TODAY()-B213-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B213)&amp;IF((TODAY()-B213)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H213" s="1" t="n"/>
@@ -5516,7 +5527,7 @@
       <c r="E214" s="25" t="n"/>
       <c r="F214" s="23" t="n"/>
       <c r="G214" s="26">
-        <f>IF(OR(B214="",E214=""),"",IF(F214&lt;&gt;"","✓ Paid",IF(TODAY()-B214&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B214-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B214)&amp;" day(s)")))</f>
+        <f>IF(OR(B214="",E214=""),"",IF(F214&lt;&gt;"","Paid",IF((TODAY()-B214)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B214-Settings!$C$10)&amp;IF((TODAY()-B214-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B214)&amp;IF((TODAY()-B214)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H214" s="1" t="n"/>
@@ -5529,7 +5540,7 @@
       <c r="E215" s="25" t="n"/>
       <c r="F215" s="23" t="n"/>
       <c r="G215" s="26">
-        <f>IF(OR(B215="",E215=""),"",IF(F215&lt;&gt;"","✓ Paid",IF(TODAY()-B215&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B215-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B215)&amp;" day(s)")))</f>
+        <f>IF(OR(B215="",E215=""),"",IF(F215&lt;&gt;"","Paid",IF((TODAY()-B215)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B215-Settings!$C$10)&amp;IF((TODAY()-B215-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B215)&amp;IF((TODAY()-B215)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H215" s="1" t="n"/>
@@ -5542,7 +5553,7 @@
       <c r="E216" s="25" t="n"/>
       <c r="F216" s="23" t="n"/>
       <c r="G216" s="26">
-        <f>IF(OR(B216="",E216=""),"",IF(F216&lt;&gt;"","✓ Paid",IF(TODAY()-B216&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B216-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B216)&amp;" day(s)")))</f>
+        <f>IF(OR(B216="",E216=""),"",IF(F216&lt;&gt;"","Paid",IF((TODAY()-B216)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B216-Settings!$C$10)&amp;IF((TODAY()-B216-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B216)&amp;IF((TODAY()-B216)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H216" s="1" t="n"/>
@@ -5555,7 +5566,7 @@
       <c r="E217" s="25" t="n"/>
       <c r="F217" s="23" t="n"/>
       <c r="G217" s="26">
-        <f>IF(OR(B217="",E217=""),"",IF(F217&lt;&gt;"","✓ Paid",IF(TODAY()-B217&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B217-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B217)&amp;" day(s)")))</f>
+        <f>IF(OR(B217="",E217=""),"",IF(F217&lt;&gt;"","Paid",IF((TODAY()-B217)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B217-Settings!$C$10)&amp;IF((TODAY()-B217-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B217)&amp;IF((TODAY()-B217)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H217" s="1" t="n"/>
@@ -5568,7 +5579,7 @@
       <c r="E218" s="25" t="n"/>
       <c r="F218" s="23" t="n"/>
       <c r="G218" s="26">
-        <f>IF(OR(B218="",E218=""),"",IF(F218&lt;&gt;"","✓ Paid",IF(TODAY()-B218&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B218-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B218)&amp;" day(s)")))</f>
+        <f>IF(OR(B218="",E218=""),"",IF(F218&lt;&gt;"","Paid",IF((TODAY()-B218)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B218-Settings!$C$10)&amp;IF((TODAY()-B218-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B218)&amp;IF((TODAY()-B218)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H218" s="1" t="n"/>
@@ -5581,7 +5592,7 @@
       <c r="E219" s="25" t="n"/>
       <c r="F219" s="23" t="n"/>
       <c r="G219" s="26">
-        <f>IF(OR(B219="",E219=""),"",IF(F219&lt;&gt;"","✓ Paid",IF(TODAY()-B219&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B219-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B219)&amp;" day(s)")))</f>
+        <f>IF(OR(B219="",E219=""),"",IF(F219&lt;&gt;"","Paid",IF((TODAY()-B219)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B219-Settings!$C$10)&amp;IF((TODAY()-B219-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B219)&amp;IF((TODAY()-B219)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H219" s="1" t="n"/>
@@ -5594,7 +5605,7 @@
       <c r="E220" s="25" t="n"/>
       <c r="F220" s="23" t="n"/>
       <c r="G220" s="26">
-        <f>IF(OR(B220="",E220=""),"",IF(F220&lt;&gt;"","✓ Paid",IF(TODAY()-B220&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B220-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B220)&amp;" day(s)")))</f>
+        <f>IF(OR(B220="",E220=""),"",IF(F220&lt;&gt;"","Paid",IF((TODAY()-B220)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B220-Settings!$C$10)&amp;IF((TODAY()-B220-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B220)&amp;IF((TODAY()-B220)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H220" s="1" t="n"/>
@@ -5607,7 +5618,7 @@
       <c r="E221" s="25" t="n"/>
       <c r="F221" s="23" t="n"/>
       <c r="G221" s="26">
-        <f>IF(OR(B221="",E221=""),"",IF(F221&lt;&gt;"","✓ Paid",IF(TODAY()-B221&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B221-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B221)&amp;" day(s)")))</f>
+        <f>IF(OR(B221="",E221=""),"",IF(F221&lt;&gt;"","Paid",IF((TODAY()-B221)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B221-Settings!$C$10)&amp;IF((TODAY()-B221-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B221)&amp;IF((TODAY()-B221)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H221" s="1" t="n"/>
@@ -5620,7 +5631,7 @@
       <c r="E222" s="25" t="n"/>
       <c r="F222" s="23" t="n"/>
       <c r="G222" s="26">
-        <f>IF(OR(B222="",E222=""),"",IF(F222&lt;&gt;"","✓ Paid",IF(TODAY()-B222&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B222-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B222)&amp;" day(s)")))</f>
+        <f>IF(OR(B222="",E222=""),"",IF(F222&lt;&gt;"","Paid",IF((TODAY()-B222)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B222-Settings!$C$10)&amp;IF((TODAY()-B222-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B222)&amp;IF((TODAY()-B222)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H222" s="1" t="n"/>
@@ -5633,7 +5644,7 @@
       <c r="E223" s="25" t="n"/>
       <c r="F223" s="23" t="n"/>
       <c r="G223" s="26">
-        <f>IF(OR(B223="",E223=""),"",IF(F223&lt;&gt;"","✓ Paid",IF(TODAY()-B223&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B223-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B223)&amp;" day(s)")))</f>
+        <f>IF(OR(B223="",E223=""),"",IF(F223&lt;&gt;"","Paid",IF((TODAY()-B223)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B223-Settings!$C$10)&amp;IF((TODAY()-B223-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B223)&amp;IF((TODAY()-B223)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H223" s="1" t="n"/>
@@ -5646,7 +5657,7 @@
       <c r="E224" s="25" t="n"/>
       <c r="F224" s="23" t="n"/>
       <c r="G224" s="26">
-        <f>IF(OR(B224="",E224=""),"",IF(F224&lt;&gt;"","✓ Paid",IF(TODAY()-B224&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B224-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B224)&amp;" day(s)")))</f>
+        <f>IF(OR(B224="",E224=""),"",IF(F224&lt;&gt;"","Paid",IF((TODAY()-B224)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B224-Settings!$C$10)&amp;IF((TODAY()-B224-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B224)&amp;IF((TODAY()-B224)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H224" s="1" t="n"/>
@@ -5659,7 +5670,7 @@
       <c r="E225" s="25" t="n"/>
       <c r="F225" s="23" t="n"/>
       <c r="G225" s="26">
-        <f>IF(OR(B225="",E225=""),"",IF(F225&lt;&gt;"","✓ Paid",IF(TODAY()-B225&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B225-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B225)&amp;" day(s)")))</f>
+        <f>IF(OR(B225="",E225=""),"",IF(F225&lt;&gt;"","Paid",IF((TODAY()-B225)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B225-Settings!$C$10)&amp;IF((TODAY()-B225-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B225)&amp;IF((TODAY()-B225)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H225" s="1" t="n"/>
@@ -5672,7 +5683,7 @@
       <c r="E226" s="25" t="n"/>
       <c r="F226" s="23" t="n"/>
       <c r="G226" s="26">
-        <f>IF(OR(B226="",E226=""),"",IF(F226&lt;&gt;"","✓ Paid",IF(TODAY()-B226&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B226-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B226)&amp;" day(s)")))</f>
+        <f>IF(OR(B226="",E226=""),"",IF(F226&lt;&gt;"","Paid",IF((TODAY()-B226)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B226-Settings!$C$10)&amp;IF((TODAY()-B226-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B226)&amp;IF((TODAY()-B226)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H226" s="1" t="n"/>
@@ -5685,7 +5696,7 @@
       <c r="E227" s="25" t="n"/>
       <c r="F227" s="23" t="n"/>
       <c r="G227" s="26">
-        <f>IF(OR(B227="",E227=""),"",IF(F227&lt;&gt;"","✓ Paid",IF(TODAY()-B227&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B227-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B227)&amp;" day(s)")))</f>
+        <f>IF(OR(B227="",E227=""),"",IF(F227&lt;&gt;"","Paid",IF((TODAY()-B227)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B227-Settings!$C$10)&amp;IF((TODAY()-B227-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B227)&amp;IF((TODAY()-B227)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H227" s="1" t="n"/>
@@ -5698,7 +5709,7 @@
       <c r="E228" s="25" t="n"/>
       <c r="F228" s="23" t="n"/>
       <c r="G228" s="26">
-        <f>IF(OR(B228="",E228=""),"",IF(F228&lt;&gt;"","✓ Paid",IF(TODAY()-B228&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B228-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B228)&amp;" day(s)")))</f>
+        <f>IF(OR(B228="",E228=""),"",IF(F228&lt;&gt;"","Paid",IF((TODAY()-B228)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B228-Settings!$C$10)&amp;IF((TODAY()-B228-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B228)&amp;IF((TODAY()-B228)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H228" s="1" t="n"/>
@@ -5711,7 +5722,7 @@
       <c r="E229" s="25" t="n"/>
       <c r="F229" s="23" t="n"/>
       <c r="G229" s="26">
-        <f>IF(OR(B229="",E229=""),"",IF(F229&lt;&gt;"","✓ Paid",IF(TODAY()-B229&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B229-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B229)&amp;" day(s)")))</f>
+        <f>IF(OR(B229="",E229=""),"",IF(F229&lt;&gt;"","Paid",IF((TODAY()-B229)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B229-Settings!$C$10)&amp;IF((TODAY()-B229-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B229)&amp;IF((TODAY()-B229)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H229" s="1" t="n"/>
@@ -5724,7 +5735,7 @@
       <c r="E230" s="25" t="n"/>
       <c r="F230" s="23" t="n"/>
       <c r="G230" s="26">
-        <f>IF(OR(B230="",E230=""),"",IF(F230&lt;&gt;"","✓ Paid",IF(TODAY()-B230&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B230-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B230)&amp;" day(s)")))</f>
+        <f>IF(OR(B230="",E230=""),"",IF(F230&lt;&gt;"","Paid",IF((TODAY()-B230)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B230-Settings!$C$10)&amp;IF((TODAY()-B230-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B230)&amp;IF((TODAY()-B230)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H230" s="1" t="n"/>
@@ -5737,7 +5748,7 @@
       <c r="E231" s="25" t="n"/>
       <c r="F231" s="23" t="n"/>
       <c r="G231" s="26">
-        <f>IF(OR(B231="",E231=""),"",IF(F231&lt;&gt;"","✓ Paid",IF(TODAY()-B231&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B231-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B231)&amp;" day(s)")))</f>
+        <f>IF(OR(B231="",E231=""),"",IF(F231&lt;&gt;"","Paid",IF((TODAY()-B231)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B231-Settings!$C$10)&amp;IF((TODAY()-B231-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B231)&amp;IF((TODAY()-B231)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H231" s="1" t="n"/>
@@ -5750,7 +5761,7 @@
       <c r="E232" s="25" t="n"/>
       <c r="F232" s="23" t="n"/>
       <c r="G232" s="26">
-        <f>IF(OR(B232="",E232=""),"",IF(F232&lt;&gt;"","✓ Paid",IF(TODAY()-B232&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B232-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B232)&amp;" day(s)")))</f>
+        <f>IF(OR(B232="",E232=""),"",IF(F232&lt;&gt;"","Paid",IF((TODAY()-B232)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B232-Settings!$C$10)&amp;IF((TODAY()-B232-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B232)&amp;IF((TODAY()-B232)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H232" s="1" t="n"/>
@@ -5763,7 +5774,7 @@
       <c r="E233" s="25" t="n"/>
       <c r="F233" s="23" t="n"/>
       <c r="G233" s="26">
-        <f>IF(OR(B233="",E233=""),"",IF(F233&lt;&gt;"","✓ Paid",IF(TODAY()-B233&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B233-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B233)&amp;" day(s)")))</f>
+        <f>IF(OR(B233="",E233=""),"",IF(F233&lt;&gt;"","Paid",IF((TODAY()-B233)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B233-Settings!$C$10)&amp;IF((TODAY()-B233-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B233)&amp;IF((TODAY()-B233)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H233" s="1" t="n"/>
@@ -5776,7 +5787,7 @@
       <c r="E234" s="25" t="n"/>
       <c r="F234" s="23" t="n"/>
       <c r="G234" s="26">
-        <f>IF(OR(B234="",E234=""),"",IF(F234&lt;&gt;"","✓ Paid",IF(TODAY()-B234&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B234-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B234)&amp;" day(s)")))</f>
+        <f>IF(OR(B234="",E234=""),"",IF(F234&lt;&gt;"","Paid",IF((TODAY()-B234)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B234-Settings!$C$10)&amp;IF((TODAY()-B234-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B234)&amp;IF((TODAY()-B234)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H234" s="1" t="n"/>
@@ -5789,7 +5800,7 @@
       <c r="E235" s="25" t="n"/>
       <c r="F235" s="23" t="n"/>
       <c r="G235" s="26">
-        <f>IF(OR(B235="",E235=""),"",IF(F235&lt;&gt;"","✓ Paid",IF(TODAY()-B235&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B235-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B235)&amp;" day(s)")))</f>
+        <f>IF(OR(B235="",E235=""),"",IF(F235&lt;&gt;"","Paid",IF((TODAY()-B235)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B235-Settings!$C$10)&amp;IF((TODAY()-B235-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B235)&amp;IF((TODAY()-B235)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H235" s="1" t="n"/>
@@ -5802,7 +5813,7 @@
       <c r="E236" s="25" t="n"/>
       <c r="F236" s="23" t="n"/>
       <c r="G236" s="26">
-        <f>IF(OR(B236="",E236=""),"",IF(F236&lt;&gt;"","✓ Paid",IF(TODAY()-B236&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B236-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B236)&amp;" day(s)")))</f>
+        <f>IF(OR(B236="",E236=""),"",IF(F236&lt;&gt;"","Paid",IF((TODAY()-B236)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B236-Settings!$C$10)&amp;IF((TODAY()-B236-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B236)&amp;IF((TODAY()-B236)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H236" s="1" t="n"/>
@@ -5815,7 +5826,7 @@
       <c r="E237" s="25" t="n"/>
       <c r="F237" s="23" t="n"/>
       <c r="G237" s="26">
-        <f>IF(OR(B237="",E237=""),"",IF(F237&lt;&gt;"","✓ Paid",IF(TODAY()-B237&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B237-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B237)&amp;" day(s)")))</f>
+        <f>IF(OR(B237="",E237=""),"",IF(F237&lt;&gt;"","Paid",IF((TODAY()-B237)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B237-Settings!$C$10)&amp;IF((TODAY()-B237-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B237)&amp;IF((TODAY()-B237)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H237" s="1" t="n"/>
@@ -5828,7 +5839,7 @@
       <c r="E238" s="25" t="n"/>
       <c r="F238" s="23" t="n"/>
       <c r="G238" s="26">
-        <f>IF(OR(B238="",E238=""),"",IF(F238&lt;&gt;"","✓ Paid",IF(TODAY()-B238&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B238-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B238)&amp;" day(s)")))</f>
+        <f>IF(OR(B238="",E238=""),"",IF(F238&lt;&gt;"","Paid",IF((TODAY()-B238)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B238-Settings!$C$10)&amp;IF((TODAY()-B238-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B238)&amp;IF((TODAY()-B238)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H238" s="1" t="n"/>
@@ -5841,7 +5852,7 @@
       <c r="E239" s="25" t="n"/>
       <c r="F239" s="23" t="n"/>
       <c r="G239" s="26">
-        <f>IF(OR(B239="",E239=""),"",IF(F239&lt;&gt;"","✓ Paid",IF(TODAY()-B239&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B239-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B239)&amp;" day(s)")))</f>
+        <f>IF(OR(B239="",E239=""),"",IF(F239&lt;&gt;"","Paid",IF((TODAY()-B239)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B239-Settings!$C$10)&amp;IF((TODAY()-B239-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B239)&amp;IF((TODAY()-B239)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H239" s="1" t="n"/>
@@ -5854,7 +5865,7 @@
       <c r="E240" s="25" t="n"/>
       <c r="F240" s="23" t="n"/>
       <c r="G240" s="26">
-        <f>IF(OR(B240="",E240=""),"",IF(F240&lt;&gt;"","✓ Paid",IF(TODAY()-B240&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B240-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B240)&amp;" day(s)")))</f>
+        <f>IF(OR(B240="",E240=""),"",IF(F240&lt;&gt;"","Paid",IF((TODAY()-B240)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B240-Settings!$C$10)&amp;IF((TODAY()-B240-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B240)&amp;IF((TODAY()-B240)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H240" s="1" t="n"/>
@@ -5867,7 +5878,7 @@
       <c r="E241" s="25" t="n"/>
       <c r="F241" s="23" t="n"/>
       <c r="G241" s="26">
-        <f>IF(OR(B241="",E241=""),"",IF(F241&lt;&gt;"","✓ Paid",IF(TODAY()-B241&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B241-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B241)&amp;" day(s)")))</f>
+        <f>IF(OR(B241="",E241=""),"",IF(F241&lt;&gt;"","Paid",IF((TODAY()-B241)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B241-Settings!$C$10)&amp;IF((TODAY()-B241-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B241)&amp;IF((TODAY()-B241)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H241" s="1" t="n"/>
@@ -5880,7 +5891,7 @@
       <c r="E242" s="25" t="n"/>
       <c r="F242" s="23" t="n"/>
       <c r="G242" s="26">
-        <f>IF(OR(B242="",E242=""),"",IF(F242&lt;&gt;"","✓ Paid",IF(TODAY()-B242&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B242-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B242)&amp;" day(s)")))</f>
+        <f>IF(OR(B242="",E242=""),"",IF(F242&lt;&gt;"","Paid",IF((TODAY()-B242)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B242-Settings!$C$10)&amp;IF((TODAY()-B242-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B242)&amp;IF((TODAY()-B242)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H242" s="1" t="n"/>
@@ -5893,7 +5904,7 @@
       <c r="E243" s="25" t="n"/>
       <c r="F243" s="23" t="n"/>
       <c r="G243" s="26">
-        <f>IF(OR(B243="",E243=""),"",IF(F243&lt;&gt;"","✓ Paid",IF(TODAY()-B243&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B243-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B243)&amp;" day(s)")))</f>
+        <f>IF(OR(B243="",E243=""),"",IF(F243&lt;&gt;"","Paid",IF((TODAY()-B243)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B243-Settings!$C$10)&amp;IF((TODAY()-B243-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B243)&amp;IF((TODAY()-B243)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H243" s="1" t="n"/>
@@ -5906,7 +5917,7 @@
       <c r="E244" s="25" t="n"/>
       <c r="F244" s="23" t="n"/>
       <c r="G244" s="26">
-        <f>IF(OR(B244="",E244=""),"",IF(F244&lt;&gt;"","✓ Paid",IF(TODAY()-B244&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B244-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B244)&amp;" day(s)")))</f>
+        <f>IF(OR(B244="",E244=""),"",IF(F244&lt;&gt;"","Paid",IF((TODAY()-B244)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B244-Settings!$C$10)&amp;IF((TODAY()-B244-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B244)&amp;IF((TODAY()-B244)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H244" s="1" t="n"/>
@@ -5919,7 +5930,7 @@
       <c r="E245" s="25" t="n"/>
       <c r="F245" s="23" t="n"/>
       <c r="G245" s="26">
-        <f>IF(OR(B245="",E245=""),"",IF(F245&lt;&gt;"","✓ Paid",IF(TODAY()-B245&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B245-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B245)&amp;" day(s)")))</f>
+        <f>IF(OR(B245="",E245=""),"",IF(F245&lt;&gt;"","Paid",IF((TODAY()-B245)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B245-Settings!$C$10)&amp;IF((TODAY()-B245-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B245)&amp;IF((TODAY()-B245)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H245" s="1" t="n"/>
@@ -5932,7 +5943,7 @@
       <c r="E246" s="25" t="n"/>
       <c r="F246" s="23" t="n"/>
       <c r="G246" s="26">
-        <f>IF(OR(B246="",E246=""),"",IF(F246&lt;&gt;"","✓ Paid",IF(TODAY()-B246&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B246-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B246)&amp;" day(s)")))</f>
+        <f>IF(OR(B246="",E246=""),"",IF(F246&lt;&gt;"","Paid",IF((TODAY()-B246)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B246-Settings!$C$10)&amp;IF((TODAY()-B246-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B246)&amp;IF((TODAY()-B246)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H246" s="1" t="n"/>
@@ -5945,7 +5956,7 @@
       <c r="E247" s="25" t="n"/>
       <c r="F247" s="23" t="n"/>
       <c r="G247" s="26">
-        <f>IF(OR(B247="",E247=""),"",IF(F247&lt;&gt;"","✓ Paid",IF(TODAY()-B247&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B247-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B247)&amp;" day(s)")))</f>
+        <f>IF(OR(B247="",E247=""),"",IF(F247&lt;&gt;"","Paid",IF((TODAY()-B247)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B247-Settings!$C$10)&amp;IF((TODAY()-B247-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B247)&amp;IF((TODAY()-B247)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H247" s="1" t="n"/>
@@ -5958,7 +5969,7 @@
       <c r="E248" s="25" t="n"/>
       <c r="F248" s="23" t="n"/>
       <c r="G248" s="26">
-        <f>IF(OR(B248="",E248=""),"",IF(F248&lt;&gt;"","✓ Paid",IF(TODAY()-B248&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B248-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B248)&amp;" day(s)")))</f>
+        <f>IF(OR(B248="",E248=""),"",IF(F248&lt;&gt;"","Paid",IF((TODAY()-B248)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B248-Settings!$C$10)&amp;IF((TODAY()-B248-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B248)&amp;IF((TODAY()-B248)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H248" s="1" t="n"/>
@@ -5971,7 +5982,7 @@
       <c r="E249" s="25" t="n"/>
       <c r="F249" s="23" t="n"/>
       <c r="G249" s="26">
-        <f>IF(OR(B249="",E249=""),"",IF(F249&lt;&gt;"","✓ Paid",IF(TODAY()-B249&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B249-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B249)&amp;" day(s)")))</f>
+        <f>IF(OR(B249="",E249=""),"",IF(F249&lt;&gt;"","Paid",IF((TODAY()-B249)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B249-Settings!$C$10)&amp;IF((TODAY()-B249-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B249)&amp;IF((TODAY()-B249)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H249" s="1" t="n"/>
@@ -5984,7 +5995,7 @@
       <c r="E250" s="25" t="n"/>
       <c r="F250" s="23" t="n"/>
       <c r="G250" s="26">
-        <f>IF(OR(B250="",E250=""),"",IF(F250&lt;&gt;"","✓ Paid",IF(TODAY()-B250&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B250-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B250)&amp;" day(s)")))</f>
+        <f>IF(OR(B250="",E250=""),"",IF(F250&lt;&gt;"","Paid",IF((TODAY()-B250)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B250-Settings!$C$10)&amp;IF((TODAY()-B250-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B250)&amp;IF((TODAY()-B250)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H250" s="1" t="n"/>
@@ -5997,7 +6008,7 @@
       <c r="E251" s="25" t="n"/>
       <c r="F251" s="23" t="n"/>
       <c r="G251" s="26">
-        <f>IF(OR(B251="",E251=""),"",IF(F251&lt;&gt;"","✓ Paid",IF(TODAY()-B251&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B251-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B251)&amp;" day(s)")))</f>
+        <f>IF(OR(B251="",E251=""),"",IF(F251&lt;&gt;"","Paid",IF((TODAY()-B251)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B251-Settings!$C$10)&amp;IF((TODAY()-B251-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B251)&amp;IF((TODAY()-B251)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H251" s="1" t="n"/>
@@ -6010,7 +6021,7 @@
       <c r="E252" s="25" t="n"/>
       <c r="F252" s="23" t="n"/>
       <c r="G252" s="26">
-        <f>IF(OR(B252="",E252=""),"",IF(F252&lt;&gt;"","✓ Paid",IF(TODAY()-B252&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B252-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B252)&amp;" day(s)")))</f>
+        <f>IF(OR(B252="",E252=""),"",IF(F252&lt;&gt;"","Paid",IF((TODAY()-B252)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B252-Settings!$C$10)&amp;IF((TODAY()-B252-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B252)&amp;IF((TODAY()-B252)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H252" s="1" t="n"/>
@@ -6023,7 +6034,7 @@
       <c r="E253" s="25" t="n"/>
       <c r="F253" s="23" t="n"/>
       <c r="G253" s="26">
-        <f>IF(OR(B253="",E253=""),"",IF(F253&lt;&gt;"","✓ Paid",IF(TODAY()-B253&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B253-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B253)&amp;" day(s)")))</f>
+        <f>IF(OR(B253="",E253=""),"",IF(F253&lt;&gt;"","Paid",IF((TODAY()-B253)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B253-Settings!$C$10)&amp;IF((TODAY()-B253-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B253)&amp;IF((TODAY()-B253)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H253" s="1" t="n"/>
@@ -6036,7 +6047,7 @@
       <c r="E254" s="25" t="n"/>
       <c r="F254" s="23" t="n"/>
       <c r="G254" s="26">
-        <f>IF(OR(B254="",E254=""),"",IF(F254&lt;&gt;"","✓ Paid",IF(TODAY()-B254&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B254-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B254)&amp;" day(s)")))</f>
+        <f>IF(OR(B254="",E254=""),"",IF(F254&lt;&gt;"","Paid",IF((TODAY()-B254)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B254-Settings!$C$10)&amp;IF((TODAY()-B254-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B254)&amp;IF((TODAY()-B254)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H254" s="1" t="n"/>
@@ -6049,7 +6060,7 @@
       <c r="E255" s="25" t="n"/>
       <c r="F255" s="23" t="n"/>
       <c r="G255" s="26">
-        <f>IF(OR(B255="",E255=""),"",IF(F255&lt;&gt;"","✓ Paid",IF(TODAY()-B255&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B255-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B255)&amp;" day(s)")))</f>
+        <f>IF(OR(B255="",E255=""),"",IF(F255&lt;&gt;"","Paid",IF((TODAY()-B255)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B255-Settings!$C$10)&amp;IF((TODAY()-B255-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B255)&amp;IF((TODAY()-B255)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H255" s="1" t="n"/>
@@ -6062,7 +6073,7 @@
       <c r="E256" s="25" t="n"/>
       <c r="F256" s="23" t="n"/>
       <c r="G256" s="26">
-        <f>IF(OR(B256="",E256=""),"",IF(F256&lt;&gt;"","✓ Paid",IF(TODAY()-B256&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B256-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B256)&amp;" day(s)")))</f>
+        <f>IF(OR(B256="",E256=""),"",IF(F256&lt;&gt;"","Paid",IF((TODAY()-B256)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B256-Settings!$C$10)&amp;IF((TODAY()-B256-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B256)&amp;IF((TODAY()-B256)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H256" s="1" t="n"/>
@@ -6075,7 +6086,7 @@
       <c r="E257" s="25" t="n"/>
       <c r="F257" s="23" t="n"/>
       <c r="G257" s="26">
-        <f>IF(OR(B257="",E257=""),"",IF(F257&lt;&gt;"","✓ Paid",IF(TODAY()-B257&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B257-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B257)&amp;" day(s)")))</f>
+        <f>IF(OR(B257="",E257=""),"",IF(F257&lt;&gt;"","Paid",IF((TODAY()-B257)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B257-Settings!$C$10)&amp;IF((TODAY()-B257-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B257)&amp;IF((TODAY()-B257)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H257" s="1" t="n"/>
@@ -6088,7 +6099,7 @@
       <c r="E258" s="25" t="n"/>
       <c r="F258" s="23" t="n"/>
       <c r="G258" s="26">
-        <f>IF(OR(B258="",E258=""),"",IF(F258&lt;&gt;"","✓ Paid",IF(TODAY()-B258&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B258-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B258)&amp;" day(s)")))</f>
+        <f>IF(OR(B258="",E258=""),"",IF(F258&lt;&gt;"","Paid",IF((TODAY()-B258)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B258-Settings!$C$10)&amp;IF((TODAY()-B258-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B258)&amp;IF((TODAY()-B258)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H258" s="1" t="n"/>
@@ -6101,7 +6112,7 @@
       <c r="E259" s="25" t="n"/>
       <c r="F259" s="23" t="n"/>
       <c r="G259" s="26">
-        <f>IF(OR(B259="",E259=""),"",IF(F259&lt;&gt;"","✓ Paid",IF(TODAY()-B259&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B259-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B259)&amp;" day(s)")))</f>
+        <f>IF(OR(B259="",E259=""),"",IF(F259&lt;&gt;"","Paid",IF((TODAY()-B259)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B259-Settings!$C$10)&amp;IF((TODAY()-B259-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B259)&amp;IF((TODAY()-B259)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H259" s="1" t="n"/>
@@ -6114,7 +6125,7 @@
       <c r="E260" s="25" t="n"/>
       <c r="F260" s="23" t="n"/>
       <c r="G260" s="26">
-        <f>IF(OR(B260="",E260=""),"",IF(F260&lt;&gt;"","✓ Paid",IF(TODAY()-B260&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B260-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B260)&amp;" day(s)")))</f>
+        <f>IF(OR(B260="",E260=""),"",IF(F260&lt;&gt;"","Paid",IF((TODAY()-B260)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B260-Settings!$C$10)&amp;IF((TODAY()-B260-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B260)&amp;IF((TODAY()-B260)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H260" s="1" t="n"/>
@@ -6127,7 +6138,7 @@
       <c r="E261" s="25" t="n"/>
       <c r="F261" s="23" t="n"/>
       <c r="G261" s="26">
-        <f>IF(OR(B261="",E261=""),"",IF(F261&lt;&gt;"","✓ Paid",IF(TODAY()-B261&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B261-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B261)&amp;" day(s)")))</f>
+        <f>IF(OR(B261="",E261=""),"",IF(F261&lt;&gt;"","Paid",IF((TODAY()-B261)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B261-Settings!$C$10)&amp;IF((TODAY()-B261-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B261)&amp;IF((TODAY()-B261)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H261" s="1" t="n"/>
@@ -6140,7 +6151,7 @@
       <c r="E262" s="25" t="n"/>
       <c r="F262" s="23" t="n"/>
       <c r="G262" s="26">
-        <f>IF(OR(B262="",E262=""),"",IF(F262&lt;&gt;"","✓ Paid",IF(TODAY()-B262&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B262-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B262)&amp;" day(s)")))</f>
+        <f>IF(OR(B262="",E262=""),"",IF(F262&lt;&gt;"","Paid",IF((TODAY()-B262)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B262-Settings!$C$10)&amp;IF((TODAY()-B262-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B262)&amp;IF((TODAY()-B262)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H262" s="1" t="n"/>
@@ -6153,7 +6164,7 @@
       <c r="E263" s="25" t="n"/>
       <c r="F263" s="23" t="n"/>
       <c r="G263" s="26">
-        <f>IF(OR(B263="",E263=""),"",IF(F263&lt;&gt;"","✓ Paid",IF(TODAY()-B263&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B263-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B263)&amp;" day(s)")))</f>
+        <f>IF(OR(B263="",E263=""),"",IF(F263&lt;&gt;"","Paid",IF((TODAY()-B263)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B263-Settings!$C$10)&amp;IF((TODAY()-B263-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B263)&amp;IF((TODAY()-B263)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H263" s="1" t="n"/>
@@ -6166,7 +6177,7 @@
       <c r="E264" s="25" t="n"/>
       <c r="F264" s="23" t="n"/>
       <c r="G264" s="26">
-        <f>IF(OR(B264="",E264=""),"",IF(F264&lt;&gt;"","✓ Paid",IF(TODAY()-B264&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B264-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B264)&amp;" day(s)")))</f>
+        <f>IF(OR(B264="",E264=""),"",IF(F264&lt;&gt;"","Paid",IF((TODAY()-B264)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B264-Settings!$C$10)&amp;IF((TODAY()-B264-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B264)&amp;IF((TODAY()-B264)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H264" s="1" t="n"/>
@@ -6179,7 +6190,7 @@
       <c r="E265" s="25" t="n"/>
       <c r="F265" s="23" t="n"/>
       <c r="G265" s="26">
-        <f>IF(OR(B265="",E265=""),"",IF(F265&lt;&gt;"","✓ Paid",IF(TODAY()-B265&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B265-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B265)&amp;" day(s)")))</f>
+        <f>IF(OR(B265="",E265=""),"",IF(F265&lt;&gt;"","Paid",IF((TODAY()-B265)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B265-Settings!$C$10)&amp;IF((TODAY()-B265-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B265)&amp;IF((TODAY()-B265)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H265" s="1" t="n"/>
@@ -6192,7 +6203,7 @@
       <c r="E266" s="25" t="n"/>
       <c r="F266" s="23" t="n"/>
       <c r="G266" s="26">
-        <f>IF(OR(B266="",E266=""),"",IF(F266&lt;&gt;"","✓ Paid",IF(TODAY()-B266&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B266-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B266)&amp;" day(s)")))</f>
+        <f>IF(OR(B266="",E266=""),"",IF(F266&lt;&gt;"","Paid",IF((TODAY()-B266)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B266-Settings!$C$10)&amp;IF((TODAY()-B266-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B266)&amp;IF((TODAY()-B266)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H266" s="1" t="n"/>
@@ -6205,7 +6216,7 @@
       <c r="E267" s="25" t="n"/>
       <c r="F267" s="23" t="n"/>
       <c r="G267" s="26">
-        <f>IF(OR(B267="",E267=""),"",IF(F267&lt;&gt;"","✓ Paid",IF(TODAY()-B267&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B267-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B267)&amp;" day(s)")))</f>
+        <f>IF(OR(B267="",E267=""),"",IF(F267&lt;&gt;"","Paid",IF((TODAY()-B267)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B267-Settings!$C$10)&amp;IF((TODAY()-B267-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B267)&amp;IF((TODAY()-B267)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H267" s="1" t="n"/>
@@ -6218,7 +6229,7 @@
       <c r="E268" s="25" t="n"/>
       <c r="F268" s="23" t="n"/>
       <c r="G268" s="26">
-        <f>IF(OR(B268="",E268=""),"",IF(F268&lt;&gt;"","✓ Paid",IF(TODAY()-B268&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B268-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B268)&amp;" day(s)")))</f>
+        <f>IF(OR(B268="",E268=""),"",IF(F268&lt;&gt;"","Paid",IF((TODAY()-B268)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B268-Settings!$C$10)&amp;IF((TODAY()-B268-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B268)&amp;IF((TODAY()-B268)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H268" s="1" t="n"/>
@@ -6231,7 +6242,7 @@
       <c r="E269" s="25" t="n"/>
       <c r="F269" s="23" t="n"/>
       <c r="G269" s="26">
-        <f>IF(OR(B269="",E269=""),"",IF(F269&lt;&gt;"","✓ Paid",IF(TODAY()-B269&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B269-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B269)&amp;" day(s)")))</f>
+        <f>IF(OR(B269="",E269=""),"",IF(F269&lt;&gt;"","Paid",IF((TODAY()-B269)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B269-Settings!$C$10)&amp;IF((TODAY()-B269-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B269)&amp;IF((TODAY()-B269)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H269" s="1" t="n"/>
@@ -6244,7 +6255,7 @@
       <c r="E270" s="25" t="n"/>
       <c r="F270" s="23" t="n"/>
       <c r="G270" s="26">
-        <f>IF(OR(B270="",E270=""),"",IF(F270&lt;&gt;"","✓ Paid",IF(TODAY()-B270&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B270-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B270)&amp;" day(s)")))</f>
+        <f>IF(OR(B270="",E270=""),"",IF(F270&lt;&gt;"","Paid",IF((TODAY()-B270)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B270-Settings!$C$10)&amp;IF((TODAY()-B270-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B270)&amp;IF((TODAY()-B270)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H270" s="1" t="n"/>
@@ -6257,7 +6268,7 @@
       <c r="E271" s="25" t="n"/>
       <c r="F271" s="23" t="n"/>
       <c r="G271" s="26">
-        <f>IF(OR(B271="",E271=""),"",IF(F271&lt;&gt;"","✓ Paid",IF(TODAY()-B271&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B271-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B271)&amp;" day(s)")))</f>
+        <f>IF(OR(B271="",E271=""),"",IF(F271&lt;&gt;"","Paid",IF((TODAY()-B271)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B271-Settings!$C$10)&amp;IF((TODAY()-B271-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B271)&amp;IF((TODAY()-B271)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H271" s="1" t="n"/>
@@ -6270,7 +6281,7 @@
       <c r="E272" s="25" t="n"/>
       <c r="F272" s="23" t="n"/>
       <c r="G272" s="26">
-        <f>IF(OR(B272="",E272=""),"",IF(F272&lt;&gt;"","✓ Paid",IF(TODAY()-B272&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B272-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B272)&amp;" day(s)")))</f>
+        <f>IF(OR(B272="",E272=""),"",IF(F272&lt;&gt;"","Paid",IF((TODAY()-B272)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B272-Settings!$C$10)&amp;IF((TODAY()-B272-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B272)&amp;IF((TODAY()-B272)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H272" s="1" t="n"/>
@@ -6283,7 +6294,7 @@
       <c r="E273" s="25" t="n"/>
       <c r="F273" s="23" t="n"/>
       <c r="G273" s="26">
-        <f>IF(OR(B273="",E273=""),"",IF(F273&lt;&gt;"","✓ Paid",IF(TODAY()-B273&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B273-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B273)&amp;" day(s)")))</f>
+        <f>IF(OR(B273="",E273=""),"",IF(F273&lt;&gt;"","Paid",IF((TODAY()-B273)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B273-Settings!$C$10)&amp;IF((TODAY()-B273-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B273)&amp;IF((TODAY()-B273)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H273" s="1" t="n"/>
@@ -6296,7 +6307,7 @@
       <c r="E274" s="25" t="n"/>
       <c r="F274" s="23" t="n"/>
       <c r="G274" s="26">
-        <f>IF(OR(B274="",E274=""),"",IF(F274&lt;&gt;"","✓ Paid",IF(TODAY()-B274&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B274-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B274)&amp;" day(s)")))</f>
+        <f>IF(OR(B274="",E274=""),"",IF(F274&lt;&gt;"","Paid",IF((TODAY()-B274)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B274-Settings!$C$10)&amp;IF((TODAY()-B274-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B274)&amp;IF((TODAY()-B274)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H274" s="1" t="n"/>
@@ -6309,7 +6320,7 @@
       <c r="E275" s="25" t="n"/>
       <c r="F275" s="23" t="n"/>
       <c r="G275" s="26">
-        <f>IF(OR(B275="",E275=""),"",IF(F275&lt;&gt;"","✓ Paid",IF(TODAY()-B275&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B275-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B275)&amp;" day(s)")))</f>
+        <f>IF(OR(B275="",E275=""),"",IF(F275&lt;&gt;"","Paid",IF((TODAY()-B275)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B275-Settings!$C$10)&amp;IF((TODAY()-B275-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B275)&amp;IF((TODAY()-B275)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H275" s="1" t="n"/>
@@ -6322,7 +6333,7 @@
       <c r="E276" s="25" t="n"/>
       <c r="F276" s="23" t="n"/>
       <c r="G276" s="26">
-        <f>IF(OR(B276="",E276=""),"",IF(F276&lt;&gt;"","✓ Paid",IF(TODAY()-B276&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B276-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B276)&amp;" day(s)")))</f>
+        <f>IF(OR(B276="",E276=""),"",IF(F276&lt;&gt;"","Paid",IF((TODAY()-B276)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B276-Settings!$C$10)&amp;IF((TODAY()-B276-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B276)&amp;IF((TODAY()-B276)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H276" s="1" t="n"/>
@@ -6335,7 +6346,7 @@
       <c r="E277" s="25" t="n"/>
       <c r="F277" s="23" t="n"/>
       <c r="G277" s="26">
-        <f>IF(OR(B277="",E277=""),"",IF(F277&lt;&gt;"","✓ Paid",IF(TODAY()-B277&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B277-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B277)&amp;" day(s)")))</f>
+        <f>IF(OR(B277="",E277=""),"",IF(F277&lt;&gt;"","Paid",IF((TODAY()-B277)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B277-Settings!$C$10)&amp;IF((TODAY()-B277-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B277)&amp;IF((TODAY()-B277)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H277" s="1" t="n"/>
@@ -6348,7 +6359,7 @@
       <c r="E278" s="25" t="n"/>
       <c r="F278" s="23" t="n"/>
       <c r="G278" s="26">
-        <f>IF(OR(B278="",E278=""),"",IF(F278&lt;&gt;"","✓ Paid",IF(TODAY()-B278&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B278-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B278)&amp;" day(s)")))</f>
+        <f>IF(OR(B278="",E278=""),"",IF(F278&lt;&gt;"","Paid",IF((TODAY()-B278)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B278-Settings!$C$10)&amp;IF((TODAY()-B278-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B278)&amp;IF((TODAY()-B278)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H278" s="1" t="n"/>
@@ -6361,7 +6372,7 @@
       <c r="E279" s="25" t="n"/>
       <c r="F279" s="23" t="n"/>
       <c r="G279" s="26">
-        <f>IF(OR(B279="",E279=""),"",IF(F279&lt;&gt;"","✓ Paid",IF(TODAY()-B279&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B279-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B279)&amp;" day(s)")))</f>
+        <f>IF(OR(B279="",E279=""),"",IF(F279&lt;&gt;"","Paid",IF((TODAY()-B279)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B279-Settings!$C$10)&amp;IF((TODAY()-B279-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B279)&amp;IF((TODAY()-B279)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H279" s="1" t="n"/>
@@ -6374,7 +6385,7 @@
       <c r="E280" s="25" t="n"/>
       <c r="F280" s="23" t="n"/>
       <c r="G280" s="26">
-        <f>IF(OR(B280="",E280=""),"",IF(F280&lt;&gt;"","✓ Paid",IF(TODAY()-B280&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B280-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B280)&amp;" day(s)")))</f>
+        <f>IF(OR(B280="",E280=""),"",IF(F280&lt;&gt;"","Paid",IF((TODAY()-B280)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B280-Settings!$C$10)&amp;IF((TODAY()-B280-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B280)&amp;IF((TODAY()-B280)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H280" s="1" t="n"/>
@@ -6387,7 +6398,7 @@
       <c r="E281" s="25" t="n"/>
       <c r="F281" s="23" t="n"/>
       <c r="G281" s="26">
-        <f>IF(OR(B281="",E281=""),"",IF(F281&lt;&gt;"","✓ Paid",IF(TODAY()-B281&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B281-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B281)&amp;" day(s)")))</f>
+        <f>IF(OR(B281="",E281=""),"",IF(F281&lt;&gt;"","Paid",IF((TODAY()-B281)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B281-Settings!$C$10)&amp;IF((TODAY()-B281-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B281)&amp;IF((TODAY()-B281)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H281" s="1" t="n"/>
@@ -6400,7 +6411,7 @@
       <c r="E282" s="25" t="n"/>
       <c r="F282" s="23" t="n"/>
       <c r="G282" s="26">
-        <f>IF(OR(B282="",E282=""),"",IF(F282&lt;&gt;"","✓ Paid",IF(TODAY()-B282&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B282-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B282)&amp;" day(s)")))</f>
+        <f>IF(OR(B282="",E282=""),"",IF(F282&lt;&gt;"","Paid",IF((TODAY()-B282)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B282-Settings!$C$10)&amp;IF((TODAY()-B282-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B282)&amp;IF((TODAY()-B282)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H282" s="1" t="n"/>
@@ -6413,7 +6424,7 @@
       <c r="E283" s="25" t="n"/>
       <c r="F283" s="23" t="n"/>
       <c r="G283" s="26">
-        <f>IF(OR(B283="",E283=""),"",IF(F283&lt;&gt;"","✓ Paid",IF(TODAY()-B283&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B283-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B283)&amp;" day(s)")))</f>
+        <f>IF(OR(B283="",E283=""),"",IF(F283&lt;&gt;"","Paid",IF((TODAY()-B283)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B283-Settings!$C$10)&amp;IF((TODAY()-B283-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B283)&amp;IF((TODAY()-B283)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H283" s="1" t="n"/>
@@ -6426,7 +6437,7 @@
       <c r="E284" s="25" t="n"/>
       <c r="F284" s="23" t="n"/>
       <c r="G284" s="26">
-        <f>IF(OR(B284="",E284=""),"",IF(F284&lt;&gt;"","✓ Paid",IF(TODAY()-B284&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B284-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B284)&amp;" day(s)")))</f>
+        <f>IF(OR(B284="",E284=""),"",IF(F284&lt;&gt;"","Paid",IF((TODAY()-B284)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B284-Settings!$C$10)&amp;IF((TODAY()-B284-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B284)&amp;IF((TODAY()-B284)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H284" s="1" t="n"/>
@@ -6439,7 +6450,7 @@
       <c r="E285" s="25" t="n"/>
       <c r="F285" s="23" t="n"/>
       <c r="G285" s="26">
-        <f>IF(OR(B285="",E285=""),"",IF(F285&lt;&gt;"","✓ Paid",IF(TODAY()-B285&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B285-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B285)&amp;" day(s)")))</f>
+        <f>IF(OR(B285="",E285=""),"",IF(F285&lt;&gt;"","Paid",IF((TODAY()-B285)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B285-Settings!$C$10)&amp;IF((TODAY()-B285-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B285)&amp;IF((TODAY()-B285)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H285" s="1" t="n"/>
@@ -6452,7 +6463,7 @@
       <c r="E286" s="25" t="n"/>
       <c r="F286" s="23" t="n"/>
       <c r="G286" s="26">
-        <f>IF(OR(B286="",E286=""),"",IF(F286&lt;&gt;"","✓ Paid",IF(TODAY()-B286&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B286-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B286)&amp;" day(s)")))</f>
+        <f>IF(OR(B286="",E286=""),"",IF(F286&lt;&gt;"","Paid",IF((TODAY()-B286)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B286-Settings!$C$10)&amp;IF((TODAY()-B286-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B286)&amp;IF((TODAY()-B286)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H286" s="1" t="n"/>
@@ -6465,7 +6476,7 @@
       <c r="E287" s="25" t="n"/>
       <c r="F287" s="23" t="n"/>
       <c r="G287" s="26">
-        <f>IF(OR(B287="",E287=""),"",IF(F287&lt;&gt;"","✓ Paid",IF(TODAY()-B287&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B287-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B287)&amp;" day(s)")))</f>
+        <f>IF(OR(B287="",E287=""),"",IF(F287&lt;&gt;"","Paid",IF((TODAY()-B287)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B287-Settings!$C$10)&amp;IF((TODAY()-B287-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B287)&amp;IF((TODAY()-B287)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H287" s="1" t="n"/>
@@ -6478,7 +6489,7 @@
       <c r="E288" s="25" t="n"/>
       <c r="F288" s="23" t="n"/>
       <c r="G288" s="26">
-        <f>IF(OR(B288="",E288=""),"",IF(F288&lt;&gt;"","✓ Paid",IF(TODAY()-B288&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B288-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B288)&amp;" day(s)")))</f>
+        <f>IF(OR(B288="",E288=""),"",IF(F288&lt;&gt;"","Paid",IF((TODAY()-B288)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B288-Settings!$C$10)&amp;IF((TODAY()-B288-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B288)&amp;IF((TODAY()-B288)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H288" s="1" t="n"/>
@@ -6491,7 +6502,7 @@
       <c r="E289" s="25" t="n"/>
       <c r="F289" s="23" t="n"/>
       <c r="G289" s="26">
-        <f>IF(OR(B289="",E289=""),"",IF(F289&lt;&gt;"","✓ Paid",IF(TODAY()-B289&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B289-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B289)&amp;" day(s)")))</f>
+        <f>IF(OR(B289="",E289=""),"",IF(F289&lt;&gt;"","Paid",IF((TODAY()-B289)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B289-Settings!$C$10)&amp;IF((TODAY()-B289-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B289)&amp;IF((TODAY()-B289)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H289" s="1" t="n"/>
@@ -6504,7 +6515,7 @@
       <c r="E290" s="25" t="n"/>
       <c r="F290" s="23" t="n"/>
       <c r="G290" s="26">
-        <f>IF(OR(B290="",E290=""),"",IF(F290&lt;&gt;"","✓ Paid",IF(TODAY()-B290&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B290-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B290)&amp;" day(s)")))</f>
+        <f>IF(OR(B290="",E290=""),"",IF(F290&lt;&gt;"","Paid",IF((TODAY()-B290)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B290-Settings!$C$10)&amp;IF((TODAY()-B290-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B290)&amp;IF((TODAY()-B290)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H290" s="1" t="n"/>
@@ -6517,7 +6528,7 @@
       <c r="E291" s="25" t="n"/>
       <c r="F291" s="23" t="n"/>
       <c r="G291" s="26">
-        <f>IF(OR(B291="",E291=""),"",IF(F291&lt;&gt;"","✓ Paid",IF(TODAY()-B291&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B291-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B291)&amp;" day(s)")))</f>
+        <f>IF(OR(B291="",E291=""),"",IF(F291&lt;&gt;"","Paid",IF((TODAY()-B291)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B291-Settings!$C$10)&amp;IF((TODAY()-B291-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B291)&amp;IF((TODAY()-B291)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H291" s="1" t="n"/>
@@ -6530,7 +6541,7 @@
       <c r="E292" s="25" t="n"/>
       <c r="F292" s="23" t="n"/>
       <c r="G292" s="26">
-        <f>IF(OR(B292="",E292=""),"",IF(F292&lt;&gt;"","✓ Paid",IF(TODAY()-B292&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B292-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B292)&amp;" day(s)")))</f>
+        <f>IF(OR(B292="",E292=""),"",IF(F292&lt;&gt;"","Paid",IF((TODAY()-B292)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B292-Settings!$C$10)&amp;IF((TODAY()-B292-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B292)&amp;IF((TODAY()-B292)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H292" s="1" t="n"/>
@@ -6543,7 +6554,7 @@
       <c r="E293" s="25" t="n"/>
       <c r="F293" s="23" t="n"/>
       <c r="G293" s="26">
-        <f>IF(OR(B293="",E293=""),"",IF(F293&lt;&gt;"","✓ Paid",IF(TODAY()-B293&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B293-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B293)&amp;" day(s)")))</f>
+        <f>IF(OR(B293="",E293=""),"",IF(F293&lt;&gt;"","Paid",IF((TODAY()-B293)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B293-Settings!$C$10)&amp;IF((TODAY()-B293-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B293)&amp;IF((TODAY()-B293)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H293" s="1" t="n"/>
@@ -6556,7 +6567,7 @@
       <c r="E294" s="25" t="n"/>
       <c r="F294" s="23" t="n"/>
       <c r="G294" s="26">
-        <f>IF(OR(B294="",E294=""),"",IF(F294&lt;&gt;"","✓ Paid",IF(TODAY()-B294&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B294-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B294)&amp;" day(s)")))</f>
+        <f>IF(OR(B294="",E294=""),"",IF(F294&lt;&gt;"","Paid",IF((TODAY()-B294)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B294-Settings!$C$10)&amp;IF((TODAY()-B294-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B294)&amp;IF((TODAY()-B294)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H294" s="1" t="n"/>
@@ -6569,7 +6580,7 @@
       <c r="E295" s="25" t="n"/>
       <c r="F295" s="23" t="n"/>
       <c r="G295" s="26">
-        <f>IF(OR(B295="",E295=""),"",IF(F295&lt;&gt;"","✓ Paid",IF(TODAY()-B295&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B295-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B295)&amp;" day(s)")))</f>
+        <f>IF(OR(B295="",E295=""),"",IF(F295&lt;&gt;"","Paid",IF((TODAY()-B295)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B295-Settings!$C$10)&amp;IF((TODAY()-B295-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B295)&amp;IF((TODAY()-B295)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H295" s="1" t="n"/>
@@ -6582,7 +6593,7 @@
       <c r="E296" s="25" t="n"/>
       <c r="F296" s="23" t="n"/>
       <c r="G296" s="26">
-        <f>IF(OR(B296="",E296=""),"",IF(F296&lt;&gt;"","✓ Paid",IF(TODAY()-B296&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B296-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B296)&amp;" day(s)")))</f>
+        <f>IF(OR(B296="",E296=""),"",IF(F296&lt;&gt;"","Paid",IF((TODAY()-B296)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B296-Settings!$C$10)&amp;IF((TODAY()-B296-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B296)&amp;IF((TODAY()-B296)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H296" s="1" t="n"/>
@@ -6595,7 +6606,7 @@
       <c r="E297" s="25" t="n"/>
       <c r="F297" s="23" t="n"/>
       <c r="G297" s="26">
-        <f>IF(OR(B297="",E297=""),"",IF(F297&lt;&gt;"","✓ Paid",IF(TODAY()-B297&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B297-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B297)&amp;" day(s)")))</f>
+        <f>IF(OR(B297="",E297=""),"",IF(F297&lt;&gt;"","Paid",IF((TODAY()-B297)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B297-Settings!$C$10)&amp;IF((TODAY()-B297-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B297)&amp;IF((TODAY()-B297)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H297" s="1" t="n"/>
@@ -6608,7 +6619,7 @@
       <c r="E298" s="25" t="n"/>
       <c r="F298" s="23" t="n"/>
       <c r="G298" s="26">
-        <f>IF(OR(B298="",E298=""),"",IF(F298&lt;&gt;"","✓ Paid",IF(TODAY()-B298&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B298-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B298)&amp;" day(s)")))</f>
+        <f>IF(OR(B298="",E298=""),"",IF(F298&lt;&gt;"","Paid",IF((TODAY()-B298)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B298-Settings!$C$10)&amp;IF((TODAY()-B298-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B298)&amp;IF((TODAY()-B298)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H298" s="1" t="n"/>
@@ -6621,7 +6632,7 @@
       <c r="E299" s="25" t="n"/>
       <c r="F299" s="23" t="n"/>
       <c r="G299" s="26">
-        <f>IF(OR(B299="",E299=""),"",IF(F299&lt;&gt;"","✓ Paid",IF(TODAY()-B299&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B299-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B299)&amp;" day(s)")))</f>
+        <f>IF(OR(B299="",E299=""),"",IF(F299&lt;&gt;"","Paid",IF((TODAY()-B299)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B299-Settings!$C$10)&amp;IF((TODAY()-B299-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B299)&amp;IF((TODAY()-B299)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H299" s="1" t="n"/>
@@ -6634,7 +6645,7 @@
       <c r="E300" s="25" t="n"/>
       <c r="F300" s="23" t="n"/>
       <c r="G300" s="26">
-        <f>IF(OR(B300="",E300=""),"",IF(F300&lt;&gt;"","✓ Paid",IF(TODAY()-B300&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B300-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B300)&amp;" day(s)")))</f>
+        <f>IF(OR(B300="",E300=""),"",IF(F300&lt;&gt;"","Paid",IF((TODAY()-B300)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B300-Settings!$C$10)&amp;IF((TODAY()-B300-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B300)&amp;IF((TODAY()-B300)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H300" s="1" t="n"/>
@@ -6647,7 +6658,7 @@
       <c r="E301" s="25" t="n"/>
       <c r="F301" s="23" t="n"/>
       <c r="G301" s="26">
-        <f>IF(OR(B301="",E301=""),"",IF(F301&lt;&gt;"","✓ Paid",IF(TODAY()-B301&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B301-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B301)&amp;" day(s)")))</f>
+        <f>IF(OR(B301="",E301=""),"",IF(F301&lt;&gt;"","Paid",IF((TODAY()-B301)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B301-Settings!$C$10)&amp;IF((TODAY()-B301-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B301)&amp;IF((TODAY()-B301)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H301" s="1" t="n"/>
@@ -6660,7 +6671,7 @@
       <c r="E302" s="25" t="n"/>
       <c r="F302" s="23" t="n"/>
       <c r="G302" s="26">
-        <f>IF(OR(B302="",E302=""),"",IF(F302&lt;&gt;"","✓ Paid",IF(TODAY()-B302&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B302-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B302)&amp;" day(s)")))</f>
+        <f>IF(OR(B302="",E302=""),"",IF(F302&lt;&gt;"","Paid",IF((TODAY()-B302)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B302-Settings!$C$10)&amp;IF((TODAY()-B302-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B302)&amp;IF((TODAY()-B302)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H302" s="1" t="n"/>
@@ -6673,7 +6684,7 @@
       <c r="E303" s="25" t="n"/>
       <c r="F303" s="23" t="n"/>
       <c r="G303" s="26">
-        <f>IF(OR(B303="",E303=""),"",IF(F303&lt;&gt;"","✓ Paid",IF(TODAY()-B303&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B303-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B303)&amp;" day(s)")))</f>
+        <f>IF(OR(B303="",E303=""),"",IF(F303&lt;&gt;"","Paid",IF((TODAY()-B303)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B303-Settings!$C$10)&amp;IF((TODAY()-B303-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B303)&amp;IF((TODAY()-B303)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H303" s="1" t="n"/>
@@ -6686,7 +6697,7 @@
       <c r="E304" s="25" t="n"/>
       <c r="F304" s="23" t="n"/>
       <c r="G304" s="26">
-        <f>IF(OR(B304="",E304=""),"",IF(F304&lt;&gt;"","✓ Paid",IF(TODAY()-B304&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B304-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B304)&amp;" day(s)")))</f>
+        <f>IF(OR(B304="",E304=""),"",IF(F304&lt;&gt;"","Paid",IF((TODAY()-B304)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B304-Settings!$C$10)&amp;IF((TODAY()-B304-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B304)&amp;IF((TODAY()-B304)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H304" s="1" t="n"/>
@@ -6699,7 +6710,7 @@
       <c r="E305" s="25" t="n"/>
       <c r="F305" s="23" t="n"/>
       <c r="G305" s="26">
-        <f>IF(OR(B305="",E305=""),"",IF(F305&lt;&gt;"","✓ Paid",IF(TODAY()-B305&gt;Settings!$C$10,"⚠ Overdue "&amp;(TODAY()-B305-Settings!$C$10)&amp;" day(s)","Waiting "&amp;(TODAY()-B305)&amp;" day(s)")))</f>
+        <f>IF(OR(B305="",E305=""),"",IF(F305&lt;&gt;"","Paid",IF((TODAY()-B305)&gt;Settings!$C$10,"Overdue by "&amp;(TODAY()-B305-Settings!$C$10)&amp;IF((TODAY()-B305-Settings!$C$10)=1," day"," days"),"Waiting "&amp;(TODAY()-B305)&amp;IF((TODAY()-B305)=1," day"," days"))))</f>
         <v/>
       </c>
       <c r="H305" s="1" t="n"/>
@@ -6717,10 +6728,10 @@
   </sheetData>
   <conditionalFormatting sqref="G6:G305">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>LEFT($G6,1)="✓"</formula>
+      <formula>$G6="Paid"</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="1">
-      <formula>LEFT($G6,1)="⚠"</formula>
+      <formula>LEFT($G6,7)="Overdue"</formula>
     </cfRule>
     <cfRule type="expression" priority="3" dxfId="2">
       <formula>LEFT($G6,7)="Waiting"</formula>
@@ -6777,7 +6788,7 @@
       <c r="A3" s="1" t="n"/>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Keep the receipt: tick 'Receipt?' when you have it.</t>
+          <t>Keep your receipts. Choose Yes under 'Receipt?' once you have it.</t>
         </is>
       </c>
       <c r="C3" s="1" t="n"/>
@@ -6849,8 +6860,10 @@
       <c r="E6" s="25" t="n">
         <v>180</v>
       </c>
-      <c r="F6" s="24" t="b">
-        <v>1</v>
+      <c r="F6" s="24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
       </c>
       <c r="G6" s="22" t="inlineStr"/>
       <c r="H6" s="1" t="n"/>
@@ -6873,8 +6886,10 @@
       <c r="E7" s="25" t="n">
         <v>96</v>
       </c>
-      <c r="F7" s="24" t="b">
-        <v>1</v>
+      <c r="F7" s="24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
       </c>
       <c r="G7" s="22" t="inlineStr">
         <is>
@@ -6901,8 +6916,10 @@
       <c r="E8" s="25" t="n">
         <v>239</v>
       </c>
-      <c r="F8" s="24" t="b">
-        <v>1</v>
+      <c r="F8" s="24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
       </c>
       <c r="G8" s="22" t="inlineStr"/>
       <c r="H8" s="1" t="n"/>
@@ -6925,8 +6942,10 @@
       <c r="E9" s="25" t="n">
         <v>86.40000000000001</v>
       </c>
-      <c r="F9" s="24" t="b">
-        <v>1</v>
+      <c r="F9" s="24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
       </c>
       <c r="G9" s="22" t="inlineStr"/>
       <c r="H9" s="1" t="n"/>
@@ -6949,8 +6968,10 @@
       <c r="E10" s="25" t="n">
         <v>19.99</v>
       </c>
-      <c r="F10" s="24" t="b">
-        <v>1</v>
+      <c r="F10" s="24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
       </c>
       <c r="G10" s="22" t="inlineStr">
         <is>
@@ -6977,12 +6998,14 @@
       <c r="E11" s="25" t="n">
         <v>329</v>
       </c>
-      <c r="F11" s="24" t="b">
-        <v>0</v>
+      <c r="F11" s="24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="G11" s="22" t="inlineStr">
         <is>
-          <t>find the invoice!</t>
+          <t>receipt missing</t>
         </is>
       </c>
       <c r="H11" s="1" t="n"/>
@@ -7005,8 +7028,10 @@
       <c r="E12" s="25" t="n">
         <v>75</v>
       </c>
-      <c r="F12" s="24" t="b">
-        <v>1</v>
+      <c r="F12" s="24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
       </c>
       <c r="G12" s="22" t="inlineStr"/>
       <c r="H12" s="1" t="n"/>
@@ -7029,8 +7054,10 @@
       <c r="E13" s="25" t="n">
         <v>120</v>
       </c>
-      <c r="F13" s="24" t="b">
-        <v>1</v>
+      <c r="F13" s="24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
       </c>
       <c r="G13" s="22" t="inlineStr"/>
       <c r="H13" s="1" t="n"/>
@@ -11976,7 +12003,7 @@
       <formula1>=Settings!$B$14:$B$28</formula1>
     </dataValidation>
     <dataValidation sqref="F6:F505" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
+      <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12815,7 +12842,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Start here: 5 minutes</t>
+          <t>Start here</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -12825,7 +12852,7 @@
       <c r="A3" s="1" t="n"/>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Only type in YELLOW cells.</t>
+          <t>Type only in the yellow cells. Everything else is calculated.</t>
         </is>
       </c>
       <c r="C3" s="1" t="n"/>
@@ -12846,7 +12873,7 @@
       </c>
       <c r="C5" s="28" t="inlineStr">
         <is>
-          <t>Settings: the year, and the share of profit you put aside for tax (ask your accountant; 25-30% is cautious).</t>
+          <t>Settings: the year, and the share of profit you put aside for tax. Ask your accountant; 25 to 30% is careful.</t>
         </is>
       </c>
       <c r="D5" s="1" t="n"/>
@@ -12866,7 +12893,7 @@
       </c>
       <c r="C7" s="28" t="inlineStr">
         <is>
-          <t>Income: one line per invoice. Fill 'Paid on' when the money arrives. Late invoices turn red.</t>
+          <t>Income: one line per invoice. Fill in 'Paid on' when the money arrives. Late invoices turn red.</t>
         </is>
       </c>
       <c r="D7" s="1" t="n"/>
@@ -12886,7 +12913,7 @@
       </c>
       <c r="C9" s="28" t="inlineStr">
         <is>
-          <t>Expenses: one line per business purchase. Tick 'Receipt?' when you have the receipt.</t>
+          <t>Expenses: one line per business purchase. Choose Yes under 'Receipt?' once you have the receipt.</t>
         </is>
       </c>
       <c r="D9" s="1" t="n"/>
@@ -12906,7 +12933,7 @@
       </c>
       <c r="C11" s="28" t="inlineStr">
         <is>
-          <t>Tax Savings: each time you move money aside for tax, add a line.</t>
+          <t>Tax Savings: add a line each time you move money aside for tax.</t>
         </is>
       </c>
       <c r="D11" s="1" t="n"/>
@@ -12921,12 +12948,12 @@
       <c r="A13" s="1" t="n"/>
       <c r="B13" s="27" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C13" s="28" t="inlineStr">
         <is>
-          <t>Dashboard: profit, what to put aside, what is still missing, quarter by quarter.</t>
+          <t>The Dashboard then shows your profit, what to put aside and what is still missing, by quarter.</t>
         </is>
       </c>
       <c r="D13" s="1" t="n"/>
@@ -12954,7 +12981,7 @@
       <c r="B17" s="1" t="n"/>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>This is a tracking tool, not tax advice. Tax rules differ by country: check your rate with an accountant.</t>
+          <t>This file tracks numbers and does not give tax advice. Tax rules differ by country, so check your rate with an accountant.</t>
         </is>
       </c>
       <c r="D17" s="1" t="n"/>
@@ -12970,7 +12997,7 @@
       <c r="B19" s="1" t="n"/>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Works in Google Sheets and Microsoft Excel. Example lines show how it works: delete them and add yours.</t>
+          <t>Works in Google Sheets and Microsoft Excel. The example lines show how it works; delete them and add your own.</t>
         </is>
       </c>
       <c r="D19" s="1" t="n"/>

</xml_diff>